<commit_message>
Review-tc round 2/3, close Đã huỷ/icon-Back coverage gaps, fix Dashboard bug (323→337 TCs)
- Verify + officially score review-tc Round 2/3 (85/100 CONDITIONAL, G1 PASS)
- Fix Dashboard COUNTIFS bug causing false 100% "executed" status (real 0%)
- Sync TC-MASTER-LATEST.xlsx tabs/content with the two canonical files
- Add DOC-v1.0-05/06 source IDs (live app observation / BA-chat confirmation)
  and remap RTM + TC DOC Source columns to use them consistently
- Close "Đã huỷ" (cancelled order) coverage gaps across Hoạt động, Trang chủ,
  Bảng tin, and Đăng tin (card badge, edit-lock, feed visibility)
- Audit and add icon-Back test cases for 6 screens lacking them
- Add OPR-07 push-notification SĐT scenario + TCs, closing the RTM
  REQ-NTF-002 gap
- Add Receiver-side cancel history-log TC, closing the 3-role gap in Huỷ đơn

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0139GVK1dvUETZFCLVMkySoT
</commit_message>
<xml_diff>
--- a/03_test-cases/v1.0/fragments/TC-BANGTIN-v1.0.xlsx
+++ b/03_test-cases/v1.0/fragments/TC-BANGTIN-v1.0.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Coverage Matrix" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$6:$U$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bảng tin &amp; Chi tiết tin'!$A$6:$U$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Coverage Matrix'!$A$1:$M$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -3419,12 +3419,12 @@
       </c>
       <c r="B16" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-009</t>
+          <t>REQ-ASN-009, REQ-ORD-004</t>
         </is>
       </c>
       <c r="C16" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §D7 (OPR-08)</t>
+          <t>Quan sát thực tế app STG (QA GiangDC2, chat 2026-07-30)</t>
         </is>
       </c>
       <c r="D16" s="239" t="inlineStr">
@@ -3434,29 +3434,29 @@
       </c>
       <c r="E16" s="239" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F16" s="239" t="inlineStr">
         <is>
-          <t>Check tin quay lại "Chờ ghép" và hiện lại Bảng tin sau khi Carrier huỷ (chưa lấy hàng)</t>
+          <t>Check tin biến mất khỏi Bảng tin ngay sau khi tự động chuyển "Hết hạn"</t>
         </is>
       </c>
       <c r="G16" s="239" t="inlineStr">
         <is>
-          <t>1 đơn đang ở trạng thái "Đã ghép", Carrier CHƯA bấm "Tôi đã lấy hàng"</t>
+          <t>Tin đang ở "Chờ ghép" và hiển thị trong Bảng tin; tin vừa tự động chuyển "Hết hạn" (quá "Đến ngày" mà chưa ai ghép)</t>
         </is>
       </c>
       <c r="H16" s="239" t="inlineStr">
         <is>
-          <t>1. Mở app FoxEco bằng tài khoản Carrier đang giữ đơn, huỷ đơn ở trạng thái "Đã ghép"
-2. Đăng nhập bằng tài khoản Carrier khác, bấm tab "Bảng tin"
-3. Tìm lại tin vừa bị huỷ trong danh sách</t>
+          <t>1. Mở app FoxEco bằng tài khoản Carrier bất kỳ
+2. Bấm tab "Bảng tin" tại bottom nav
+3. Tìm lại tin vừa "Hết hạn" trong danh sách</t>
         </is>
       </c>
       <c r="I16" s="239" t="inlineStr">
         <is>
-          <t>3. Tin quay về trạng thái "Chờ ghép" và xuất hiện trở lại trong danh sách Bảng tin</t>
+          <t>3. Tin KHÔNG còn xuất hiện trong danh sách Bảng tin</t>
         </is>
       </c>
       <c r="J16" s="239" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="AP16" s="240" t="inlineStr">
         <is>
-          <t>Technique: ST-matched-posted (huỷ trước khi lấy hàng)</t>
+          <t>Technique: ST-posted-expired (hiệu ứng trên bề mặt Bảng tin) | Bổ sung 2026-07-30 theo yêu cầu user, đóng gap: `TC_06.6` chỉ cover chiều "Đã ghép", chưa cover 2 chiều rời "Chờ ghép" còn lại (Hết hạn/Đã huỷ). Đối chứng khác bề mặt với `TC_01.9` (Hoạt động, verify badge "Hết hạn" hiển thị đúng — đó là màn cá nhân, còn đây là feed công khai).</t>
         </is>
       </c>
     </row>
@@ -3525,12 +3525,12 @@
       </c>
       <c r="B17" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-009</t>
+          <t>REQ-ASN-009, REQ-CNL-001</t>
         </is>
       </c>
       <c r="C17" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §D7 (OPR-08)</t>
+          <t>Quan sát thực tế app STG (QA GiangDC2, chat 2026-07-30)</t>
         </is>
       </c>
       <c r="D17" s="239" t="inlineStr">
@@ -3540,29 +3540,29 @@
       </c>
       <c r="E17" s="239" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F17" s="239" t="inlineStr">
         <is>
-          <t>Check tin quay lại Bảng tin được Carrier khác ghép lại thành công</t>
+          <t>Check tin biến mất khỏi Bảng tin ngay sau khi bị Sender huỷ</t>
         </is>
       </c>
       <c r="G17" s="239" t="inlineStr">
         <is>
-          <t>1 tin vừa quay về "Chờ ghép" do Carrier trước đó huỷ (chưa lấy hàng), đang hiển thị lại trong Bảng tin</t>
+          <t>Tin đang ở "Chờ ghép" và hiển thị trong Bảng tin; Sender vừa huỷ tin đó (qua popup "Huỷ đơn")</t>
         </is>
       </c>
       <c r="H17" s="239" t="inlineStr">
         <is>
-          <t>1. Mở app FoxEco bằng tài khoản Carrier khác
-2. Bấm tab "Bảng tin", mở Chi tiết tin của tin vừa quay lại
-3. Bấm "Tôi mang giúp được" rồi bấm "Xác nhận" trong modal</t>
+          <t>1. Mở app FoxEco bằng tài khoản Carrier bất kỳ
+2. Bấm tab "Bảng tin" tại bottom nav
+3. Tìm lại tin vừa bị huỷ trong danh sách</t>
         </is>
       </c>
       <c r="I17" s="239" t="inlineStr">
         <is>
-          <t>3. Ghép thành công — đơn chuyển sang "Đã ghép" với Carrier mới, tin lại ẩn khỏi Bảng tin</t>
+          <t>3. Tin KHÔNG còn xuất hiện trong danh sách Bảng tin</t>
         </is>
       </c>
       <c r="J17" s="239" t="inlineStr">
@@ -3607,126 +3607,126 @@
       <c r="AK17" s="240" t="n"/>
       <c r="AL17" s="240" t="n"/>
       <c r="AM17" s="241">
-        <f>IF($A17="","",IF(OR($N17="Yes",$S17="Yes",$X17="Yes",$AC17="Yes",$AH17="Yes"),"Yes","No"))</f>
+        <f>IF($A16="","",IF(OR($N16="Yes",$S16="Yes",$X16="Yes",$AC16="Yes",$AH16="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN17" s="241">
-        <f>IF($A17="","",IFERROR(IF($AI17&lt;&gt;"",$AI17,IF($AD17&lt;&gt;"",$AD17,IF($Y17&lt;&gt;"",$Y17,IF($T17&lt;&gt;"",$T17,IF($O17&lt;&gt;"",$O17,""))))),""))</f>
+        <f>IF($A16="","",IFERROR(IF($AI16&lt;&gt;"",$AI16,IF($AD16&lt;&gt;"",$AD16,IF($Y16&lt;&gt;"",$Y16,IF($T16&lt;&gt;"",$T16,IF($O16&lt;&gt;"",$O16,""))))),""))</f>
         <v/>
       </c>
       <c r="AO17" s="241">
-        <f>IFERROR(IF($AJ17&lt;&gt;"",$AJ17,IF($AE17&lt;&gt;"",$AE17,IF($Z17&lt;&gt;"",$Z17,IF($U17&lt;&gt;"",$U17,IF($P17&lt;&gt;"",$P17,""))))),"")</f>
+        <f>IFERROR(IF($AJ16&lt;&gt;"",$AJ16,IF($AE16&lt;&gt;"",$AE16,IF($Z16&lt;&gt;"",$Z16,IF($U16&lt;&gt;"",$U16,IF($P16&lt;&gt;"",$P16,""))))),"")</f>
         <v/>
       </c>
       <c r="AP17" s="240" t="inlineStr">
         <is>
-          <t>Technique: ST-reposted-matched (khớp lại sau khi quay về POSTED)</t>
+          <t>Technique: ST-posted-cancelled (hiệu ứng trên bề mặt Bảng tin) | Bổ sung 2026-07-30 theo yêu cầu user, đóng gap tương tự TC trên. Đối chứng khác bề mặt với `TC_01.21`/`TC_05.21` (Hoạt động/Trang chủ: tin Đã huỷ vẫn hiển thị ở màn CÁ NHÂN của actor) — Bảng tin là feed CÔNG KHAI, phải biến mất ngay khi tin không còn "đang tìm người ghép".</t>
         </is>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1" s="206">
-      <c r="A18" s="244">
+      <c r="A18" s="239">
         <f>IF(C18="","",$C$2&amp;"."&amp;COUNTA($C$8:C18)&amp;"")</f>
         <v/>
       </c>
-      <c r="B18" s="243" t="inlineStr">
-        <is>
-          <t>REQ-ASN-007</t>
-        </is>
-      </c>
-      <c r="C18" s="243" t="inlineStr">
-        <is>
-          <t>DOC-v1.0-01 §D7 (OPR-04)</t>
-        </is>
-      </c>
-      <c r="D18" s="243" t="inlineStr">
+      <c r="B18" s="239" t="inlineStr">
+        <is>
+          <t>REQ-ASN-009</t>
+        </is>
+      </c>
+      <c r="C18" s="239" t="inlineStr">
+        <is>
+          <t>DOC-v1.0-01 §D7 (OPR-08)</t>
+        </is>
+      </c>
+      <c r="D18" s="239" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="E18" s="243" t="inlineStr">
+      <c r="E18" s="239" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F18" s="243" t="inlineStr">
-        <is>
-          <t>Check thứ tự tin trong Bảng tin: tin gần tuyến nhất hiển thị trước</t>
-        </is>
-      </c>
-      <c r="G18" s="243" t="inlineStr">
-        <is>
-          <t>Carrier đã đăng tuyến OFFER; Bảng tin có 3 tin NEED phù hợp với độ gần tuyến KHÁC nhau và cùng thời điểm đăng</t>
-        </is>
-      </c>
-      <c r="H18" s="243" t="inlineStr">
-        <is>
-          <t>1. Mở app FoxEco
-2. Bấm tab "Bảng tin" tại bottom nav
-3. Quan sát thứ tự các tin trong danh sách</t>
-        </is>
-      </c>
-      <c r="I18" s="243" t="inlineStr">
-        <is>
-          <t>3. Danh sách sắp xếp theo độ gần tuyến: tin gần tuyến nhất ở vị trí đầu tiên, tin xa tuyến nhất ở cuối</t>
-        </is>
-      </c>
-      <c r="J18" s="245" t="inlineStr">
+      <c r="F18" s="239" t="inlineStr">
+        <is>
+          <t>Check tin quay lại "Chờ ghép" và hiện lại Bảng tin sau khi Carrier huỷ (chưa lấy hàng)</t>
+        </is>
+      </c>
+      <c r="G18" s="239" t="inlineStr">
+        <is>
+          <t>1 đơn đang ở trạng thái "Đã ghép", Carrier CHƯA bấm "Tôi đã lấy hàng"</t>
+        </is>
+      </c>
+      <c r="H18" s="239" t="inlineStr">
+        <is>
+          <t>1. Mở app FoxEco bằng tài khoản Carrier đang giữ đơn, huỷ đơn ở trạng thái "Đã ghép"
+2. Đăng nhập bằng tài khoản Carrier khác, bấm tab "Bảng tin"
+3. Tìm lại tin vừa bị huỷ trong danh sách</t>
+        </is>
+      </c>
+      <c r="I18" s="239" t="inlineStr">
+        <is>
+          <t>3. Tin quay về trạng thái "Chờ ghép" và xuất hiện trở lại trong danh sách Bảng tin</t>
+        </is>
+      </c>
+      <c r="J18" s="239" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="K18" s="245" t="inlineStr">
+      <c r="K18" s="239" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L18" s="245" t="inlineStr">
+      <c r="L18" s="239" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M18" s="245" t="n"/>
-      <c r="N18" s="245" t="n"/>
-      <c r="O18" s="245" t="n"/>
-      <c r="P18" s="245" t="n"/>
-      <c r="Q18" s="245" t="n"/>
-      <c r="R18" s="245" t="n"/>
-      <c r="S18" s="245" t="n"/>
-      <c r="T18" s="245" t="n"/>
-      <c r="U18" s="245" t="n"/>
-      <c r="V18" s="245" t="n"/>
-      <c r="W18" s="245" t="n"/>
-      <c r="X18" s="245" t="n"/>
-      <c r="Y18" s="245" t="n"/>
-      <c r="Z18" s="245" t="n"/>
-      <c r="AA18" s="245" t="n"/>
-      <c r="AB18" s="246" t="n"/>
-      <c r="AC18" s="246" t="n"/>
-      <c r="AD18" s="246" t="n"/>
-      <c r="AE18" s="246" t="n"/>
-      <c r="AF18" s="246" t="n"/>
-      <c r="AG18" s="246" t="n"/>
-      <c r="AH18" s="246" t="n"/>
-      <c r="AI18" s="246" t="n"/>
-      <c r="AJ18" s="246" t="n"/>
-      <c r="AK18" s="246" t="n"/>
-      <c r="AL18" s="246" t="n"/>
-      <c r="AM18" s="247">
-        <f>IF($A18="","",IF(OR($N18="Yes",$S18="Yes",$X18="Yes",$AC18="Yes",$AH18="Yes"),"Yes","No"))</f>
+      <c r="M18" s="239" t="n"/>
+      <c r="N18" s="239" t="n"/>
+      <c r="O18" s="239" t="n"/>
+      <c r="P18" s="239" t="n"/>
+      <c r="Q18" s="239" t="n"/>
+      <c r="R18" s="239" t="n"/>
+      <c r="S18" s="239" t="n"/>
+      <c r="T18" s="239" t="n"/>
+      <c r="U18" s="239" t="n"/>
+      <c r="V18" s="239" t="n"/>
+      <c r="W18" s="239" t="n"/>
+      <c r="X18" s="239" t="n"/>
+      <c r="Y18" s="239" t="n"/>
+      <c r="Z18" s="239" t="n"/>
+      <c r="AA18" s="239" t="n"/>
+      <c r="AB18" s="240" t="n"/>
+      <c r="AC18" s="240" t="n"/>
+      <c r="AD18" s="240" t="n"/>
+      <c r="AE18" s="240" t="n"/>
+      <c r="AF18" s="240" t="n"/>
+      <c r="AG18" s="240" t="n"/>
+      <c r="AH18" s="240" t="n"/>
+      <c r="AI18" s="240" t="n"/>
+      <c r="AJ18" s="240" t="n"/>
+      <c r="AK18" s="240" t="n"/>
+      <c r="AL18" s="240" t="n"/>
+      <c r="AM18" s="241">
+        <f>IF($A16="","",IF(OR($N16="Yes",$S16="Yes",$X16="Yes",$AC16="Yes",$AH16="Yes"),"Yes","No"))</f>
         <v/>
       </c>
-      <c r="AN18" s="247">
-        <f>IF($A18="","",IFERROR(IF($AI18&lt;&gt;"",$AI18,IF($AD18&lt;&gt;"",$AD18,IF($Y18&lt;&gt;"",$Y18,IF($T18&lt;&gt;"",$T18,IF($O18&lt;&gt;"",$O18,""))))),""))</f>
+      <c r="AN18" s="241">
+        <f>IF($A16="","",IFERROR(IF($AI16&lt;&gt;"",$AI16,IF($AD16&lt;&gt;"",$AD16,IF($Y16&lt;&gt;"",$Y16,IF($T16&lt;&gt;"",$T16,IF($O16&lt;&gt;"",$O16,""))))),""))</f>
         <v/>
       </c>
-      <c r="AO18" s="247">
-        <f>IFERROR(IF($AJ18&lt;&gt;"",$AJ18,IF($AE18&lt;&gt;"",$AE18,IF($Z18&lt;&gt;"",$Z18,IF($U18&lt;&gt;"",$U18,IF($P18&lt;&gt;"",$P18,""))))),"")</f>
+      <c r="AO18" s="241">
+        <f>IFERROR(IF($AJ16&lt;&gt;"",$AJ16,IF($AE16&lt;&gt;"",$AE16,IF($Z16&lt;&gt;"",$Z16,IF($U16&lt;&gt;"",$U16,IF($P16&lt;&gt;"",$P16,""))))),"")</f>
         <v/>
       </c>
-      <c r="AP18" s="247" t="inlineStr">
-        <is>
-          <t>Technique: DT-rule1 (độ gần tuyến khác nhau → sắp theo độ gần) | Cần bổ sung test data trong catalog</t>
+      <c r="AP18" s="240" t="inlineStr">
+        <is>
+          <t>Technique: ST-matched-posted (huỷ trước khi lấy hàng)</t>
         </is>
       </c>
     </row>
@@ -3737,12 +3737,12 @@
       </c>
       <c r="B19" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-007</t>
+          <t>REQ-ASN-009</t>
         </is>
       </c>
       <c r="C19" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §D7 (OPR-04)</t>
+          <t>DOC-v1.0-01 §D7 (OPR-08)</t>
         </is>
       </c>
       <c r="D19" s="239" t="inlineStr">
@@ -3757,24 +3757,24 @@
       </c>
       <c r="F19" s="239" t="inlineStr">
         <is>
-          <t>Check thứ tự tin trong Bảng tin khi độ gần tuyến bằng nhau: tin đăng mới hơn hiển thị trước</t>
+          <t>Check tin quay lại Bảng tin được Carrier khác ghép lại thành công</t>
         </is>
       </c>
       <c r="G19" s="239" t="inlineStr">
         <is>
-          <t>Carrier đã đăng tuyến OFFER; Bảng tin có 2 tin NEED CÙNG độ gần tuyến nhưng thời điểm đăng khác nhau</t>
+          <t>1 tin vừa quay về "Chờ ghép" do Carrier trước đó huỷ (chưa lấy hàng), đang hiển thị lại trong Bảng tin</t>
         </is>
       </c>
       <c r="H19" s="239" t="inlineStr">
         <is>
-          <t>1. Mở app FoxEco
-2. Bấm tab "Bảng tin" tại bottom nav
-3. Quan sát thứ tự 2 tin trong danh sách</t>
+          <t>1. Mở app FoxEco bằng tài khoản Carrier khác
+2. Bấm tab "Bảng tin", mở Chi tiết tin của tin vừa quay lại
+3. Bấm "Tôi mang giúp được" rồi bấm "Xác nhận" trong modal</t>
         </is>
       </c>
       <c r="I19" s="239" t="inlineStr">
         <is>
-          <t>3. Tin có thời điểm đăng mới hơn hiển thị trước tin đăng cũ hơn</t>
+          <t>3. Ghép thành công — đơn chuyển sang "Đã ghép" với Carrier mới, tin lại ẩn khỏi Bảng tin</t>
         </is>
       </c>
       <c r="J19" s="239" t="inlineStr">
@@ -3819,116 +3819,174 @@
       <c r="AK19" s="240" t="n"/>
       <c r="AL19" s="240" t="n"/>
       <c r="AM19" s="241">
-        <f>IF($A19="","",IF(OR($N19="Yes",$S19="Yes",$X19="Yes",$AC19="Yes",$AH19="Yes"),"Yes","No"))</f>
+        <f>IF($A17="","",IF(OR($N17="Yes",$S17="Yes",$X17="Yes",$AC17="Yes",$AH17="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN19" s="241">
-        <f>IF($A19="","",IFERROR(IF($AI19&lt;&gt;"",$AI19,IF($AD19&lt;&gt;"",$AD19,IF($Y19&lt;&gt;"",$Y19,IF($T19&lt;&gt;"",$T19,IF($O19&lt;&gt;"",$O19,""))))),""))</f>
+        <f>IF($A17="","",IFERROR(IF($AI17&lt;&gt;"",$AI17,IF($AD17&lt;&gt;"",$AD17,IF($Y17&lt;&gt;"",$Y17,IF($T17&lt;&gt;"",$T17,IF($O17&lt;&gt;"",$O17,""))))),""))</f>
         <v/>
       </c>
       <c r="AO19" s="241">
-        <f>IFERROR(IF($AJ19&lt;&gt;"",$AJ19,IF($AE19&lt;&gt;"",$AE19,IF($Z19&lt;&gt;"",$Z19,IF($U19&lt;&gt;"",$U19,IF($P19&lt;&gt;"",$P19,""))))),"")</f>
+        <f>IFERROR(IF($AJ17&lt;&gt;"",$AJ17,IF($AE17&lt;&gt;"",$AE17,IF($Z17&lt;&gt;"",$Z17,IF($U17&lt;&gt;"",$U17,IF($P17&lt;&gt;"",$P17,""))))),"")</f>
         <v/>
       </c>
       <c r="AP19" s="240" t="inlineStr">
         <is>
-          <t>Technique: DT-rule2 (độ gần tuyến bằng nhau → sắp theo thời gian đăng mới nhất) | Cần bổ sung test data trong catalog</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1" s="206">
-      <c r="A20" s="231" t="n"/>
-      <c r="B20" s="232" t="inlineStr">
-        <is>
-          <t>Block Chi tiết tin — Thông tin hàng</t>
-        </is>
-      </c>
-      <c r="C20" s="211" t="n"/>
-      <c r="D20" s="211" t="n"/>
-      <c r="E20" s="211" t="n"/>
-      <c r="F20" s="211" t="n"/>
-      <c r="G20" s="211" t="n"/>
-      <c r="H20" s="211" t="n"/>
-      <c r="I20" s="209" t="n"/>
-      <c r="J20" s="231" t="n"/>
-      <c r="K20" s="231" t="n"/>
-      <c r="L20" s="231" t="n"/>
-      <c r="M20" s="231" t="n"/>
-      <c r="N20" s="235" t="n"/>
-      <c r="O20" s="235" t="n"/>
-      <c r="P20" s="235" t="n"/>
-      <c r="Q20" s="235" t="n"/>
-      <c r="R20" s="235" t="n"/>
-      <c r="S20" s="235" t="n"/>
-      <c r="T20" s="235" t="n"/>
-      <c r="U20" s="235" t="n"/>
-      <c r="V20" s="235" t="n"/>
-      <c r="W20" s="235" t="n"/>
-      <c r="X20" s="235" t="n"/>
-      <c r="Y20" s="235" t="n"/>
-      <c r="Z20" s="235" t="n"/>
-      <c r="AA20" s="235" t="n"/>
-      <c r="AB20" s="236" t="n"/>
-      <c r="AC20" s="236" t="n"/>
-      <c r="AD20" s="236" t="n"/>
-      <c r="AE20" s="236" t="n"/>
-      <c r="AF20" s="236" t="n"/>
-      <c r="AG20" s="236" t="n"/>
-      <c r="AH20" s="236" t="n"/>
-      <c r="AI20" s="236" t="n"/>
-      <c r="AJ20" s="236" t="n"/>
-      <c r="AK20" s="236" t="n"/>
-      <c r="AL20" s="236" t="n"/>
-      <c r="AM20" s="237" t="n"/>
-      <c r="AN20" s="237" t="n"/>
-      <c r="AO20" s="237" t="n"/>
-      <c r="AP20" s="238" t="n"/>
+          <t>Technique: ST-reposted-matched (khớp lại sau khi quay về POSTED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1" s="206">
+      <c r="A20" s="244">
+        <f>IF(C20="","",$C$2&amp;"."&amp;COUNTA($C$8:C20)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="B20" s="243" t="inlineStr">
+        <is>
+          <t>REQ-ASN-007</t>
+        </is>
+      </c>
+      <c r="C20" s="243" t="inlineStr">
+        <is>
+          <t>DOC-v1.0-01 §D7 (OPR-04)</t>
+        </is>
+      </c>
+      <c r="D20" s="243" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E20" s="243" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F20" s="243" t="inlineStr">
+        <is>
+          <t>Check thứ tự tin trong Bảng tin: tin gần tuyến nhất hiển thị trước</t>
+        </is>
+      </c>
+      <c r="G20" s="243" t="inlineStr">
+        <is>
+          <t>Carrier đã đăng tuyến OFFER; Bảng tin có 3 tin NEED phù hợp với độ gần tuyến KHÁC nhau và cùng thời điểm đăng</t>
+        </is>
+      </c>
+      <c r="H20" s="243" t="inlineStr">
+        <is>
+          <t>1. Mở app FoxEco
+2. Bấm tab "Bảng tin" tại bottom nav
+3. Quan sát thứ tự các tin trong danh sách</t>
+        </is>
+      </c>
+      <c r="I20" s="243" t="inlineStr">
+        <is>
+          <t>3. Danh sách sắp xếp theo độ gần tuyến: tin gần tuyến nhất ở vị trí đầu tiên, tin xa tuyến nhất ở cuối</t>
+        </is>
+      </c>
+      <c r="J20" s="245" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="K20" s="245" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L20" s="245" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M20" s="245" t="n"/>
+      <c r="N20" s="245" t="n"/>
+      <c r="O20" s="245" t="n"/>
+      <c r="P20" s="245" t="n"/>
+      <c r="Q20" s="245" t="n"/>
+      <c r="R20" s="245" t="n"/>
+      <c r="S20" s="245" t="n"/>
+      <c r="T20" s="245" t="n"/>
+      <c r="U20" s="245" t="n"/>
+      <c r="V20" s="245" t="n"/>
+      <c r="W20" s="245" t="n"/>
+      <c r="X20" s="245" t="n"/>
+      <c r="Y20" s="245" t="n"/>
+      <c r="Z20" s="245" t="n"/>
+      <c r="AA20" s="245" t="n"/>
+      <c r="AB20" s="246" t="n"/>
+      <c r="AC20" s="246" t="n"/>
+      <c r="AD20" s="246" t="n"/>
+      <c r="AE20" s="246" t="n"/>
+      <c r="AF20" s="246" t="n"/>
+      <c r="AG20" s="246" t="n"/>
+      <c r="AH20" s="246" t="n"/>
+      <c r="AI20" s="246" t="n"/>
+      <c r="AJ20" s="246" t="n"/>
+      <c r="AK20" s="246" t="n"/>
+      <c r="AL20" s="246" t="n"/>
+      <c r="AM20" s="247">
+        <f>IF($A18="","",IF(OR($N18="Yes",$S18="Yes",$X18="Yes",$AC18="Yes",$AH18="Yes"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="AN20" s="247">
+        <f>IF($A18="","",IFERROR(IF($AI18&lt;&gt;"",$AI18,IF($AD18&lt;&gt;"",$AD18,IF($Y18&lt;&gt;"",$Y18,IF($T18&lt;&gt;"",$T18,IF($O18&lt;&gt;"",$O18,""))))),""))</f>
+        <v/>
+      </c>
+      <c r="AO20" s="247">
+        <f>IFERROR(IF($AJ18&lt;&gt;"",$AJ18,IF($AE18&lt;&gt;"",$AE18,IF($Z18&lt;&gt;"",$Z18,IF($U18&lt;&gt;"",$U18,IF($P18&lt;&gt;"",$P18,""))))),"")</f>
+        <v/>
+      </c>
+      <c r="AP20" s="247" t="inlineStr">
+        <is>
+          <t>Technique: DT-rule1 (độ gần tuyến khác nhau → sắp theo độ gần) | Cần bổ sung test data trong catalog</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="60" customHeight="1" s="206">
       <c r="A21" s="239">
         <f>IF(C21="","",$C$2&amp;"."&amp;COUNTA($C$8:C21)&amp;"")</f>
         <v/>
       </c>
-      <c r="B21" s="242" t="inlineStr">
-        <is>
-          <t>REQ-ORD-001</t>
-        </is>
-      </c>
-      <c r="C21" s="243" t="inlineStr">
-        <is>
-          <t>DOC-v1.0-02 §3.4 Table 5</t>
-        </is>
-      </c>
-      <c r="D21" s="243" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="E21" s="243" t="inlineStr">
+      <c r="B21" s="239" t="inlineStr">
+        <is>
+          <t>REQ-ASN-007</t>
+        </is>
+      </c>
+      <c r="C21" s="239" t="inlineStr">
+        <is>
+          <t>DOC-v1.0-01 §D7 (OPR-04)</t>
+        </is>
+      </c>
+      <c r="D21" s="239" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E21" s="239" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F21" s="243" t="inlineStr">
-        <is>
-          <t>Check đầy đủ + đúng 3 trường hiển thị tại block "Thông tin hàng" màn Chi tiết tin</t>
-        </is>
-      </c>
-      <c r="G21" s="243" t="inlineStr">
-        <is>
-          <t>Bảng tin có ít nhất 1 tin "Chờ ghép" do người khác đăng, tin có đủ ảnh và ghi chú</t>
-        </is>
-      </c>
-      <c r="H21" s="243" t="inlineStr">
+      <c r="F21" s="239" t="inlineStr">
+        <is>
+          <t>Check thứ tự tin trong Bảng tin khi độ gần tuyến bằng nhau: tin đăng mới hơn hiển thị trước</t>
+        </is>
+      </c>
+      <c r="G21" s="239" t="inlineStr">
+        <is>
+          <t>Carrier đã đăng tuyến OFFER; Bảng tin có 2 tin NEED CÙNG độ gần tuyến nhưng thời điểm đăng khác nhau</t>
+        </is>
+      </c>
+      <c r="H21" s="239" t="inlineStr">
         <is>
           <t>1. Mở app FoxEco
-2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
-3. Quan sát block "Thông tin hàng"</t>
-        </is>
-      </c>
-      <c r="I21" s="243" t="inlineStr">
-        <is>
-          <t>3. Block "Thông tin hàng" hiển thị đủ 3 trường: (1) ảnh sản phẩm, (2) Loại hàng và Giá trị (bố cục 2 cột), (3) Ghi chú — không thiếu trường nào</t>
+2. Bấm tab "Bảng tin" tại bottom nav
+3. Quan sát thứ tự 2 tin trong danh sách</t>
+        </is>
+      </c>
+      <c r="I21" s="239" t="inlineStr">
+        <is>
+          <t>3. Tin có thời điểm đăng mới hơn hiển thị trước tin đăng cũ hơn</t>
         </is>
       </c>
       <c r="J21" s="239" t="inlineStr">
@@ -3973,128 +4031,70 @@
       <c r="AK21" s="240" t="n"/>
       <c r="AL21" s="240" t="n"/>
       <c r="AM21" s="241">
-        <f>IF($A21="","",IF(OR($N21="Yes",$S21="Yes",$X21="Yes",$AC21="Yes",$AH21="Yes"),"Yes","No"))</f>
+        <f>IF($A19="","",IF(OR($N19="Yes",$S19="Yes",$X19="Yes",$AC19="Yes",$AH19="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN21" s="241">
-        <f>IF($A21="","",IFERROR(IF($AI21&lt;&gt;"",$AI21,IF($AD21&lt;&gt;"",$AD21,IF($Y21&lt;&gt;"",$Y21,IF($T21&lt;&gt;"",$T21,IF($O21&lt;&gt;"",$O21,""))))),""))</f>
+        <f>IF($A19="","",IFERROR(IF($AI19&lt;&gt;"",$AI19,IF($AD19&lt;&gt;"",$AD19,IF($Y19&lt;&gt;"",$Y19,IF($T19&lt;&gt;"",$T19,IF($O19&lt;&gt;"",$O19,""))))),""))</f>
         <v/>
       </c>
       <c r="AO21" s="241">
-        <f>IFERROR(IF($AJ21&lt;&gt;"",$AJ21,IF($AE21&lt;&gt;"",$AE21,IF($Z21&lt;&gt;"",$Z21,IF($U21&lt;&gt;"",$U21,IF($P21&lt;&gt;"",$P21,""))))),"")</f>
+        <f>IFERROR(IF($AJ19&lt;&gt;"",$AJ19,IF($AE19&lt;&gt;"",$AE19,IF($Z19&lt;&gt;"",$Z19,IF($U19&lt;&gt;"",$U19,IF($P19&lt;&gt;"",$P19,""))))),"")</f>
         <v/>
       </c>
       <c r="AP21" s="240" t="inlineStr">
         <is>
-          <t>Field/column completeness check — auto-derived (xem generate.md Step 3b)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1" s="206">
-      <c r="A22" s="239">
-        <f>IF(C22="","",$C$2&amp;"."&amp;COUNTA($C$8:C22)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="B22" s="239" t="inlineStr">
-        <is>
-          <t>REQ-ORD-001</t>
-        </is>
-      </c>
-      <c r="C22" s="239" t="inlineStr">
-        <is>
-          <t>DOC-v1.0-02 §3.4 Table 5</t>
-        </is>
-      </c>
-      <c r="D22" s="239" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="E22" s="239" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F22" s="239" t="inlineStr">
-        <is>
-          <t>Check ảnh sản phẩm hiển thị đúng ảnh đã tải lên khi tin có kèm ảnh</t>
-        </is>
-      </c>
-      <c r="G22" s="239" t="inlineStr">
-        <is>
-          <t>Tin được đăng có kèm đúng 1 ảnh hàng hợp lệ đã biết trước nội dung — file [TBD: ảnh mẫu, vd "hang-tai-lieu.jpg" — JPG, 1.2MB], khác rõ rệt với ảnh mặc định của hệ thống</t>
-        </is>
-      </c>
-      <c r="H22" s="239" t="inlineStr">
-        <is>
-          <t>1. Mở app FoxEco
-2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
-3. Quan sát ảnh sản phẩm tại block "Thông tin hàng"</t>
-        </is>
-      </c>
-      <c r="I22" s="239" t="inlineStr">
-        <is>
-          <t>3. Ảnh sản phẩm hiển thị đúng nội dung của chính file ảnh đã tải lên lúc đăng tin (đối chiếu trực quan với file gốc ở Pre-condition), KHÔNG phải ảnh minh hoạ mặc định của hệ thống</t>
-        </is>
-      </c>
-      <c r="J22" s="239" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="K22" s="239" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L22" s="239" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M22" s="239" t="n"/>
-      <c r="N22" s="239" t="n"/>
-      <c r="O22" s="239" t="n"/>
-      <c r="P22" s="239" t="n"/>
-      <c r="Q22" s="239" t="n"/>
-      <c r="R22" s="239" t="n"/>
-      <c r="S22" s="239" t="n"/>
-      <c r="T22" s="239" t="n"/>
-      <c r="U22" s="239" t="n"/>
-      <c r="V22" s="239" t="n"/>
-      <c r="W22" s="239" t="n"/>
-      <c r="X22" s="239" t="n"/>
-      <c r="Y22" s="239" t="n"/>
-      <c r="Z22" s="239" t="n"/>
-      <c r="AA22" s="239" t="n"/>
-      <c r="AB22" s="240" t="n"/>
-      <c r="AC22" s="240" t="n"/>
-      <c r="AD22" s="240" t="n"/>
-      <c r="AE22" s="240" t="n"/>
-      <c r="AF22" s="240" t="n"/>
-      <c r="AG22" s="240" t="n"/>
-      <c r="AH22" s="240" t="n"/>
-      <c r="AI22" s="240" t="n"/>
-      <c r="AJ22" s="240" t="n"/>
-      <c r="AK22" s="240" t="n"/>
-      <c r="AL22" s="240" t="n"/>
-      <c r="AM22" s="241">
-        <f>IF($A22="","",IF(OR($N22="Yes",$S22="Yes",$X22="Yes",$AC22="Yes",$AH22="Yes"),"Yes","No"))</f>
-        <v/>
-      </c>
-      <c r="AN22" s="241">
-        <f>IF($A22="","",IFERROR(IF($AI22&lt;&gt;"",$AI22,IF($AD22&lt;&gt;"",$AD22,IF($Y22&lt;&gt;"",$Y22,IF($T22&lt;&gt;"",$T22,IF($O22&lt;&gt;"",$O22,""))))),""))</f>
-        <v/>
-      </c>
-      <c r="AO22" s="241">
-        <f>IFERROR(IF($AJ22&lt;&gt;"",$AJ22,IF($AE22&lt;&gt;"",$AE22,IF($Z22&lt;&gt;"",$Z22,IF($U22&lt;&gt;"",$U22,IF($P22&lt;&gt;"",$P22,""))))),"")</f>
-        <v/>
-      </c>
-      <c r="AP22" s="240" t="inlineStr">
-        <is>
-          <t>Technique: EP-with-image | Cần bổ sung test data trong catalog (catalog chưa có bộ ảnh hàng mẫu để đối chiếu trực quan — xem test_data_catalog.md §Fixture)</t>
-        </is>
-      </c>
+          <t>Technique: DT-rule2 (độ gần tuyến bằng nhau → sắp theo thời gian đăng mới nhất) | Cần bổ sung test data trong catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" s="206">
+      <c r="A22" s="231" t="n"/>
+      <c r="B22" s="232" t="inlineStr">
+        <is>
+          <t>Block Chi tiết tin — Thông tin hàng</t>
+        </is>
+      </c>
+      <c r="C22" s="211" t="n"/>
+      <c r="D22" s="211" t="n"/>
+      <c r="E22" s="211" t="n"/>
+      <c r="F22" s="211" t="n"/>
+      <c r="G22" s="211" t="n"/>
+      <c r="H22" s="211" t="n"/>
+      <c r="I22" s="209" t="n"/>
+      <c r="J22" s="231" t="n"/>
+      <c r="K22" s="231" t="n"/>
+      <c r="L22" s="231" t="n"/>
+      <c r="M22" s="231" t="n"/>
+      <c r="N22" s="235" t="n"/>
+      <c r="O22" s="235" t="n"/>
+      <c r="P22" s="235" t="n"/>
+      <c r="Q22" s="235" t="n"/>
+      <c r="R22" s="235" t="n"/>
+      <c r="S22" s="235" t="n"/>
+      <c r="T22" s="235" t="n"/>
+      <c r="U22" s="235" t="n"/>
+      <c r="V22" s="235" t="n"/>
+      <c r="W22" s="235" t="n"/>
+      <c r="X22" s="235" t="n"/>
+      <c r="Y22" s="235" t="n"/>
+      <c r="Z22" s="235" t="n"/>
+      <c r="AA22" s="235" t="n"/>
+      <c r="AB22" s="236" t="n"/>
+      <c r="AC22" s="236" t="n"/>
+      <c r="AD22" s="236" t="n"/>
+      <c r="AE22" s="236" t="n"/>
+      <c r="AF22" s="236" t="n"/>
+      <c r="AG22" s="236" t="n"/>
+      <c r="AH22" s="236" t="n"/>
+      <c r="AI22" s="236" t="n"/>
+      <c r="AJ22" s="236" t="n"/>
+      <c r="AK22" s="236" t="n"/>
+      <c r="AL22" s="236" t="n"/>
+      <c r="AM22" s="237" t="n"/>
+      <c r="AN22" s="237" t="n"/>
+      <c r="AO22" s="237" t="n"/>
+      <c r="AP22" s="238" t="n"/>
     </row>
     <row r="23" ht="60" customHeight="1" s="206">
       <c r="A23" s="239">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C23" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-02 §3.4 Table 5</t>
+          <t>Quan sát thực tế app STG (QA GiangDC2, chat 2026-07-30)</t>
         </is>
       </c>
       <c r="D23" s="239" t="inlineStr">
@@ -4123,24 +4123,25 @@
       </c>
       <c r="F23" s="239" t="inlineStr">
         <is>
-          <t>Check ảnh sản phẩm hiển thị ảnh mặc định khi tin không tải ảnh</t>
+          <t>Check icon quay lại tại màn Chi tiết tin</t>
         </is>
       </c>
       <c r="G23" s="239" t="inlineStr">
         <is>
-          <t>Tin được đăng KHÔNG kèm ảnh hàng nào</t>
+          <t>Bảng tin có ít nhất 1 tin ở trạng thái "Chờ ghép"</t>
         </is>
       </c>
       <c r="H23" s="239" t="inlineStr">
         <is>
           <t>1. Mở app FoxEco
-2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
-3. Quan sát ảnh sản phẩm tại block "Thông tin hàng"</t>
+2. Bấm tab "Bảng tin" tại bottom nav
+3. Bấm vào 1 card bất kỳ để mở màn Chi tiết tin
+4. Bấm icon quay lại (←) ở Header</t>
         </is>
       </c>
       <c r="I23" s="239" t="inlineStr">
         <is>
-          <t>3. Hiển thị ảnh minh hoạ mặc định của hệ thống, không để khoảng trống/lỗi render ảnh</t>
+          <t>4. Điều hướng đúng về màn Bảng tin (màn vừa mở Chi tiết tin từ đó)</t>
         </is>
       </c>
       <c r="J23" s="239" t="inlineStr">
@@ -4185,20 +4186,20 @@
       <c r="AK23" s="240" t="n"/>
       <c r="AL23" s="240" t="n"/>
       <c r="AM23" s="241">
-        <f>IF($A23="","",IF(OR($N23="Yes",$S23="Yes",$X23="Yes",$AC23="Yes",$AH23="Yes"),"Yes","No"))</f>
+        <f>IF($A19="","",IF(OR($N19="Yes",$S19="Yes",$X19="Yes",$AC19="Yes",$AH19="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN23" s="241">
-        <f>IF($A23="","",IFERROR(IF($AI23&lt;&gt;"",$AI23,IF($AD23&lt;&gt;"",$AD23,IF($Y23&lt;&gt;"",$Y23,IF($T23&lt;&gt;"",$T23,IF($O23&lt;&gt;"",$O23,""))))),""))</f>
+        <f>IF($A19="","",IFERROR(IF($AI19&lt;&gt;"",$AI19,IF($AD19&lt;&gt;"",$AD19,IF($Y19&lt;&gt;"",$Y19,IF($T19&lt;&gt;"",$T19,IF($O19&lt;&gt;"",$O19,""))))),""))</f>
         <v/>
       </c>
       <c r="AO23" s="241">
-        <f>IFERROR(IF($AJ23&lt;&gt;"",$AJ23,IF($AE23&lt;&gt;"",$AE23,IF($Z23&lt;&gt;"",$Z23,IF($U23&lt;&gt;"",$U23,IF($P23&lt;&gt;"",$P23,""))))),"")</f>
+        <f>IFERROR(IF($AJ19&lt;&gt;"",$AJ19,IF($AE19&lt;&gt;"",$AE19,IF($Z19&lt;&gt;"",$Z19,IF($U19&lt;&gt;"",$U19,IF($P19&lt;&gt;"",$P19,""))))),"")</f>
         <v/>
       </c>
       <c r="AP23" s="240" t="inlineStr">
         <is>
-          <t>Technique: EP-no-image</t>
+          <t>Technique: EP-back-icon. Bổ sung 2026-07-30 theo yêu cầu user (QA GiangDC2 xác nhận trực tiếp trên app STG: icon quay lại tồn tại và hoạt động đúng ở màn này) — phát hiện khi quét lại toàn bộ TC-MASTER, kiểm tra completeness icon Back cho từng màn hình.</t>
         </is>
       </c>
     </row>
@@ -4207,46 +4208,46 @@
         <f>IF(C24="","",$C$2&amp;"."&amp;COUNTA($C$8:C24)&amp;"")</f>
         <v/>
       </c>
-      <c r="B24" s="239" t="inlineStr">
+      <c r="B24" s="242" t="inlineStr">
         <is>
           <t>REQ-ORD-001</t>
         </is>
       </c>
-      <c r="C24" s="239" t="inlineStr">
+      <c r="C24" s="243" t="inlineStr">
         <is>
           <t>DOC-v1.0-02 §3.4 Table 5</t>
         </is>
       </c>
-      <c r="D24" s="239" t="inlineStr">
+      <c r="D24" s="243" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="E24" s="239" t="inlineStr">
+      <c r="E24" s="243" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F24" s="239" t="inlineStr">
-        <is>
-          <t>Check nội dung Chi tiết tin khớp đúng dữ liệu đã nhập lúc đăng tin</t>
-        </is>
-      </c>
-      <c r="G24" s="239" t="inlineStr">
-        <is>
-          <t>Vừa đăng 1 tin NEED với dữ liệu đã biết trước: Loại hàng "Tài liệu", Giá trị "thấp", Ghi chú "gọi trước khi tới"</t>
-        </is>
-      </c>
-      <c r="H24" s="239" t="inlineStr">
+      <c r="F24" s="243" t="inlineStr">
+        <is>
+          <t>Check đầy đủ + đúng 3 trường hiển thị tại block "Thông tin hàng" màn Chi tiết tin</t>
+        </is>
+      </c>
+      <c r="G24" s="243" t="inlineStr">
+        <is>
+          <t>Bảng tin có ít nhất 1 tin "Chờ ghép" do người khác đăng, tin có đủ ảnh và ghi chú</t>
+        </is>
+      </c>
+      <c r="H24" s="243" t="inlineStr">
         <is>
           <t>1. Mở app FoxEco
 2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
-3. Đối chiếu từng trường trên Chi tiết tin với dữ liệu đã nhập lúc đăng</t>
-        </is>
-      </c>
-      <c r="I24" s="239" t="inlineStr">
-        <is>
-          <t>3. Loại hàng hiển thị "Tài liệu", Giá trị hiển thị "thấp", Ghi chú hiển thị "gọi trước khi tới" — khớp chính xác dữ liệu đã nhập, không bị cắt/đổi</t>
+3. Quan sát block "Thông tin hàng"</t>
+        </is>
+      </c>
+      <c r="I24" s="243" t="inlineStr">
+        <is>
+          <t>3. Block "Thông tin hàng" hiển thị đủ 3 trường: (1) ảnh sản phẩm, (2) Loại hàng và Giá trị (bố cục 2 cột), (3) Ghi chú — không thiếu trường nào</t>
         </is>
       </c>
       <c r="J24" s="239" t="inlineStr">
@@ -4291,66 +4292,128 @@
       <c r="AK24" s="240" t="n"/>
       <c r="AL24" s="240" t="n"/>
       <c r="AM24" s="241">
-        <f>IF($A24="","",IF(OR($N24="Yes",$S24="Yes",$X24="Yes",$AC24="Yes",$AH24="Yes"),"Yes","No"))</f>
+        <f>IF($A21="","",IF(OR($N21="Yes",$S21="Yes",$X21="Yes",$AC21="Yes",$AH21="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN24" s="241">
-        <f>IF($A24="","",IFERROR(IF($AI24&lt;&gt;"",$AI24,IF($AD24&lt;&gt;"",$AD24,IF($Y24&lt;&gt;"",$Y24,IF($T24&lt;&gt;"",$T24,IF($O24&lt;&gt;"",$O24,""))))),""))</f>
+        <f>IF($A21="","",IFERROR(IF($AI21&lt;&gt;"",$AI21,IF($AD21&lt;&gt;"",$AD21,IF($Y21&lt;&gt;"",$Y21,IF($T21&lt;&gt;"",$T21,IF($O21&lt;&gt;"",$O21,""))))),""))</f>
         <v/>
       </c>
       <c r="AO24" s="241">
-        <f>IFERROR(IF($AJ24&lt;&gt;"",$AJ24,IF($AE24&lt;&gt;"",$AE24,IF($Z24&lt;&gt;"",$Z24,IF($U24&lt;&gt;"",$U24,IF($P24&lt;&gt;"",$P24,""))))),"")</f>
+        <f>IFERROR(IF($AJ21&lt;&gt;"",$AJ21,IF($AE21&lt;&gt;"",$AE21,IF($Z21&lt;&gt;"",$Z21,IF($U21&lt;&gt;"",$U21,IF($P21&lt;&gt;"",$P21,""))))),"")</f>
         <v/>
       </c>
-      <c r="AP24" s="240" t="n"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" s="206">
-      <c r="A25" s="231" t="n"/>
-      <c r="B25" s="248" t="inlineStr">
-        <is>
-          <t>Block Chi tiết tin — Lộ trình &amp; liên hệ</t>
-        </is>
-      </c>
-      <c r="C25" s="211" t="n"/>
-      <c r="D25" s="211" t="n"/>
-      <c r="E25" s="211" t="n"/>
-      <c r="F25" s="211" t="n"/>
-      <c r="G25" s="211" t="n"/>
-      <c r="H25" s="211" t="n"/>
-      <c r="I25" s="209" t="n"/>
-      <c r="J25" s="231" t="n"/>
-      <c r="K25" s="231" t="n"/>
-      <c r="L25" s="231" t="n"/>
-      <c r="M25" s="231" t="n"/>
-      <c r="N25" s="235" t="n"/>
-      <c r="O25" s="235" t="n"/>
-      <c r="P25" s="235" t="n"/>
-      <c r="Q25" s="235" t="n"/>
-      <c r="R25" s="235" t="n"/>
-      <c r="S25" s="235" t="n"/>
-      <c r="T25" s="235" t="n"/>
-      <c r="U25" s="235" t="n"/>
-      <c r="V25" s="235" t="n"/>
-      <c r="W25" s="235" t="n"/>
-      <c r="X25" s="235" t="n"/>
-      <c r="Y25" s="235" t="n"/>
-      <c r="Z25" s="235" t="n"/>
-      <c r="AA25" s="235" t="n"/>
-      <c r="AB25" s="236" t="n"/>
-      <c r="AC25" s="236" t="n"/>
-      <c r="AD25" s="236" t="n"/>
-      <c r="AE25" s="236" t="n"/>
-      <c r="AF25" s="236" t="n"/>
-      <c r="AG25" s="236" t="n"/>
-      <c r="AH25" s="236" t="n"/>
-      <c r="AI25" s="236" t="n"/>
-      <c r="AJ25" s="236" t="n"/>
-      <c r="AK25" s="236" t="n"/>
-      <c r="AL25" s="236" t="n"/>
-      <c r="AM25" s="237" t="n"/>
-      <c r="AN25" s="237" t="n"/>
-      <c r="AO25" s="237" t="n"/>
-      <c r="AP25" s="238" t="n"/>
+      <c r="AP24" s="240" t="inlineStr">
+        <is>
+          <t>Field/column completeness check — auto-derived (xem generate.md Step 3b)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1" s="206">
+      <c r="A25" s="239">
+        <f>IF(C25="","",$C$2&amp;"."&amp;COUNTA($C$8:C25)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="B25" s="239" t="inlineStr">
+        <is>
+          <t>REQ-ORD-001</t>
+        </is>
+      </c>
+      <c r="C25" s="239" t="inlineStr">
+        <is>
+          <t>DOC-v1.0-02 §3.4 Table 5</t>
+        </is>
+      </c>
+      <c r="D25" s="239" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E25" s="239" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F25" s="239" t="inlineStr">
+        <is>
+          <t>Check ảnh sản phẩm hiển thị đúng ảnh đã tải lên khi tin có kèm ảnh</t>
+        </is>
+      </c>
+      <c r="G25" s="239" t="inlineStr">
+        <is>
+          <t>Tin được đăng có kèm đúng 1 ảnh hàng hợp lệ đã biết trước nội dung — file [TBD: ảnh mẫu, vd "hang-tai-lieu.jpg" — JPG, 1.2MB], khác rõ rệt với ảnh mặc định của hệ thống</t>
+        </is>
+      </c>
+      <c r="H25" s="239" t="inlineStr">
+        <is>
+          <t>1. Mở app FoxEco
+2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
+3. Quan sát ảnh sản phẩm tại block "Thông tin hàng"</t>
+        </is>
+      </c>
+      <c r="I25" s="239" t="inlineStr">
+        <is>
+          <t>3. Ảnh sản phẩm hiển thị đúng nội dung của chính file ảnh đã tải lên lúc đăng tin (đối chiếu trực quan với file gốc ở Pre-condition), KHÔNG phải ảnh minh hoạ mặc định của hệ thống</t>
+        </is>
+      </c>
+      <c r="J25" s="239" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="K25" s="239" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L25" s="239" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M25" s="239" t="n"/>
+      <c r="N25" s="239" t="n"/>
+      <c r="O25" s="239" t="n"/>
+      <c r="P25" s="239" t="n"/>
+      <c r="Q25" s="239" t="n"/>
+      <c r="R25" s="239" t="n"/>
+      <c r="S25" s="239" t="n"/>
+      <c r="T25" s="239" t="n"/>
+      <c r="U25" s="239" t="n"/>
+      <c r="V25" s="239" t="n"/>
+      <c r="W25" s="239" t="n"/>
+      <c r="X25" s="239" t="n"/>
+      <c r="Y25" s="239" t="n"/>
+      <c r="Z25" s="239" t="n"/>
+      <c r="AA25" s="239" t="n"/>
+      <c r="AB25" s="240" t="n"/>
+      <c r="AC25" s="240" t="n"/>
+      <c r="AD25" s="240" t="n"/>
+      <c r="AE25" s="240" t="n"/>
+      <c r="AF25" s="240" t="n"/>
+      <c r="AG25" s="240" t="n"/>
+      <c r="AH25" s="240" t="n"/>
+      <c r="AI25" s="240" t="n"/>
+      <c r="AJ25" s="240" t="n"/>
+      <c r="AK25" s="240" t="n"/>
+      <c r="AL25" s="240" t="n"/>
+      <c r="AM25" s="241">
+        <f>IF($A22="","",IF(OR($N22="Yes",$S22="Yes",$X22="Yes",$AC22="Yes",$AH22="Yes"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="AN25" s="241">
+        <f>IF($A22="","",IFERROR(IF($AI22&lt;&gt;"",$AI22,IF($AD22&lt;&gt;"",$AD22,IF($Y22&lt;&gt;"",$Y22,IF($T22&lt;&gt;"",$T22,IF($O22&lt;&gt;"",$O22,""))))),""))</f>
+        <v/>
+      </c>
+      <c r="AO25" s="241">
+        <f>IFERROR(IF($AJ22&lt;&gt;"",$AJ22,IF($AE22&lt;&gt;"",$AE22,IF($Z22&lt;&gt;"",$Z22,IF($U22&lt;&gt;"",$U22,IF($P22&lt;&gt;"",$P22,""))))),"")</f>
+        <v/>
+      </c>
+      <c r="AP25" s="240" t="inlineStr">
+        <is>
+          <t>Technique: EP-with-image | Cần bổ sung test data trong catalog (catalog chưa có bộ ảnh hàng mẫu để đối chiếu trực quan — xem test_data_catalog.md §Fixture)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="60" customHeight="1" s="206">
       <c r="A26" s="239">
@@ -4359,7 +4422,7 @@
       </c>
       <c r="B26" s="239" t="inlineStr">
         <is>
-          <t>REQ-ORD-001, REQ-ASN-002</t>
+          <t>REQ-ORD-001</t>
         </is>
       </c>
       <c r="C26" s="239" t="inlineStr">
@@ -4374,29 +4437,29 @@
       </c>
       <c r="E26" s="239" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F26" s="239" t="inlineStr">
         <is>
-          <t>Check đầy đủ + đúng 4 nhóm thông tin tại block "Lộ trình &amp; liên hệ" màn Chi tiết tin</t>
+          <t>Check ảnh sản phẩm hiển thị ảnh mặc định khi tin không tải ảnh</t>
         </is>
       </c>
       <c r="G26" s="239" t="inlineStr">
         <is>
-          <t>Tin đang ở trạng thái "Chờ ghép", người xem là Carrier (không phải chủ tin)</t>
+          <t>Tin được đăng KHÔNG kèm ảnh hàng nào</t>
         </is>
       </c>
       <c r="H26" s="239" t="inlineStr">
         <is>
           <t>1. Mở app FoxEco
 2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
-3. Quan sát block "Lộ trình &amp; liên hệ"</t>
+3. Quan sát ảnh sản phẩm tại block "Thông tin hàng"</t>
         </is>
       </c>
       <c r="I26" s="239" t="inlineStr">
         <is>
-          <t>3. Block hiển thị đủ 4 nhóm: (1) Lộ trình gồm điểm Lấy hàng + điểm Giao hàng + khung "Bản đồ · ~X km", (2) Khung giờ mong muốn giao nhận, (3) Người gửi — hiển thị Tên (SĐT và nút "Gọi" CHƯA khả dụng khi tin còn "Chờ ghép", theo BR-CON-02/C-ASN-01), (4) nút "Tôi mang giúp được"</t>
+          <t>3. Hiển thị ảnh minh hoạ mặc định của hệ thống, không để khoảng trống/lỗi render ảnh</t>
         </is>
       </c>
       <c r="J26" s="239" t="inlineStr">
@@ -4441,20 +4504,20 @@
       <c r="AK26" s="240" t="n"/>
       <c r="AL26" s="240" t="n"/>
       <c r="AM26" s="241">
-        <f>IF($A26="","",IF(OR($N26="Yes",$S26="Yes",$X26="Yes",$AC26="Yes",$AH26="Yes"),"Yes","No"))</f>
+        <f>IF($A23="","",IF(OR($N23="Yes",$S23="Yes",$X23="Yes",$AC23="Yes",$AH23="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN26" s="241">
-        <f>IF($A26="","",IFERROR(IF($AI26&lt;&gt;"",$AI26,IF($AD26&lt;&gt;"",$AD26,IF($Y26&lt;&gt;"",$Y26,IF($T26&lt;&gt;"",$T26,IF($O26&lt;&gt;"",$O26,""))))),""))</f>
+        <f>IF($A23="","",IFERROR(IF($AI23&lt;&gt;"",$AI23,IF($AD23&lt;&gt;"",$AD23,IF($Y23&lt;&gt;"",$Y23,IF($T23&lt;&gt;"",$T23,IF($O23&lt;&gt;"",$O23,""))))),""))</f>
         <v/>
       </c>
       <c r="AO26" s="241">
-        <f>IFERROR(IF($AJ26&lt;&gt;"",$AJ26,IF($AE26&lt;&gt;"",$AE26,IF($Z26&lt;&gt;"",$Z26,IF($U26&lt;&gt;"",$U26,IF($P26&lt;&gt;"",$P26,""))))),"")</f>
+        <f>IFERROR(IF($AJ23&lt;&gt;"",$AJ23,IF($AE23&lt;&gt;"",$AE23,IF($Z23&lt;&gt;"",$Z23,IF($U23&lt;&gt;"",$U23,IF($P23&lt;&gt;"",$P23,""))))),"")</f>
         <v/>
       </c>
       <c r="AP26" s="240" t="inlineStr">
         <is>
-          <t>Field/column completeness check — auto-derived (xem generate.md Step 3b) | Trường SĐT + nút "Gọi" chỉ khả dụng SAU khi ghép (BR-CON-02, C-ASN-01 Resolved) — xem TC regression SĐT không lộ + TC lộ SĐT sau ghép</t>
+          <t>Technique: EP-no-image</t>
         </is>
       </c>
     </row>
@@ -4480,29 +4543,29 @@
       </c>
       <c r="E27" s="239" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F27" s="239" t="inlineStr">
         <is>
-          <t>Check khung "Bản đồ · ~X km" hiển thị đúng dạng placeholder tĩnh</t>
+          <t>Check nội dung Chi tiết tin khớp đúng dữ liệu đã nhập lúc đăng tin</t>
         </is>
       </c>
       <c r="G27" s="239" t="inlineStr">
         <is>
-          <t>Tin đang ở trạng thái "Chờ ghép" với 2 địa chỉ lấy/giao khác nhau</t>
+          <t>Vừa đăng 1 tin NEED với dữ liệu đã biết trước: Loại hàng "Tài liệu", Giá trị "thấp", Ghi chú "gọi trước khi tới"</t>
         </is>
       </c>
       <c r="H27" s="239" t="inlineStr">
         <is>
           <t>1. Mở app FoxEco
 2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
-3. Quan sát khung bản đồ trong block "Lộ trình &amp; liên hệ" và thử bấm vào khung đó</t>
+3. Đối chiếu từng trường trên Chi tiết tin với dữ liệu đã nhập lúc đăng</t>
         </is>
       </c>
       <c r="I27" s="239" t="inlineStr">
         <is>
-          <t>3. Khung hiển thị đúng dạng text "Bản đồ · ~[N] km"; đây là placeholder tĩnh — bấm vào KHÔNG mở bản đồ thật, không phát sinh điều hướng</t>
+          <t>3. Loại hàng hiển thị "Tài liệu", Giá trị hiển thị "thấp", Ghi chú hiển thị "gọi trước khi tới" — khớp chính xác dữ liệu đã nhập, không bị cắt/đổi</t>
         </is>
       </c>
       <c r="J27" s="239" t="inlineStr">
@@ -4547,172 +4610,172 @@
       <c r="AK27" s="240" t="n"/>
       <c r="AL27" s="240" t="n"/>
       <c r="AM27" s="241">
-        <f>IF($A27="","",IF(OR($N27="Yes",$S27="Yes",$X27="Yes",$AC27="Yes",$AH27="Yes"),"Yes","No"))</f>
+        <f>IF($A24="","",IF(OR($N24="Yes",$S24="Yes",$X24="Yes",$AC24="Yes",$AH24="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN27" s="241">
-        <f>IF($A27="","",IFERROR(IF($AI27&lt;&gt;"",$AI27,IF($AD27&lt;&gt;"",$AD27,IF($Y27&lt;&gt;"",$Y27,IF($T27&lt;&gt;"",$T27,IF($O27&lt;&gt;"",$O27,""))))),""))</f>
+        <f>IF($A24="","",IFERROR(IF($AI24&lt;&gt;"",$AI24,IF($AD24&lt;&gt;"",$AD24,IF($Y24&lt;&gt;"",$Y24,IF($T24&lt;&gt;"",$T24,IF($O24&lt;&gt;"",$O24,""))))),""))</f>
         <v/>
       </c>
       <c r="AO27" s="241">
-        <f>IFERROR(IF($AJ27&lt;&gt;"",$AJ27,IF($AE27&lt;&gt;"",$AE27,IF($Z27&lt;&gt;"",$Z27,IF($U27&lt;&gt;"",$U27,IF($P27&lt;&gt;"",$P27,""))))),"")</f>
+        <f>IFERROR(IF($AJ24&lt;&gt;"",$AJ24,IF($AE24&lt;&gt;"",$AE24,IF($Z24&lt;&gt;"",$Z24,IF($U24&lt;&gt;"",$U24,IF($P24&lt;&gt;"",$P24,""))))),"")</f>
         <v/>
       </c>
       <c r="AP27" s="240" t="n"/>
     </row>
-    <row r="28" ht="60" customHeight="1" s="206">
-      <c r="A28" s="239">
-        <f>IF(C28="","",$C$2&amp;"."&amp;COUNTA($C$8:C28)&amp;"")</f>
+    <row r="28" ht="20" customHeight="1" s="206">
+      <c r="A28" s="231" t="n"/>
+      <c r="B28" s="248" t="inlineStr">
+        <is>
+          <t>Block Chi tiết tin — Lộ trình &amp; liên hệ</t>
+        </is>
+      </c>
+      <c r="C28" s="211" t="n"/>
+      <c r="D28" s="211" t="n"/>
+      <c r="E28" s="211" t="n"/>
+      <c r="F28" s="211" t="n"/>
+      <c r="G28" s="211" t="n"/>
+      <c r="H28" s="211" t="n"/>
+      <c r="I28" s="209" t="n"/>
+      <c r="J28" s="231" t="n"/>
+      <c r="K28" s="231" t="n"/>
+      <c r="L28" s="231" t="n"/>
+      <c r="M28" s="231" t="n"/>
+      <c r="N28" s="235" t="n"/>
+      <c r="O28" s="235" t="n"/>
+      <c r="P28" s="235" t="n"/>
+      <c r="Q28" s="235" t="n"/>
+      <c r="R28" s="235" t="n"/>
+      <c r="S28" s="235" t="n"/>
+      <c r="T28" s="235" t="n"/>
+      <c r="U28" s="235" t="n"/>
+      <c r="V28" s="235" t="n"/>
+      <c r="W28" s="235" t="n"/>
+      <c r="X28" s="235" t="n"/>
+      <c r="Y28" s="235" t="n"/>
+      <c r="Z28" s="235" t="n"/>
+      <c r="AA28" s="235" t="n"/>
+      <c r="AB28" s="236" t="n"/>
+      <c r="AC28" s="236" t="n"/>
+      <c r="AD28" s="236" t="n"/>
+      <c r="AE28" s="236" t="n"/>
+      <c r="AF28" s="236" t="n"/>
+      <c r="AG28" s="236" t="n"/>
+      <c r="AH28" s="236" t="n"/>
+      <c r="AI28" s="236" t="n"/>
+      <c r="AJ28" s="236" t="n"/>
+      <c r="AK28" s="236" t="n"/>
+      <c r="AL28" s="236" t="n"/>
+      <c r="AM28" s="237" t="n"/>
+      <c r="AN28" s="237" t="n"/>
+      <c r="AO28" s="237" t="n"/>
+      <c r="AP28" s="238" t="n"/>
+    </row>
+    <row r="29" ht="60" customHeight="1" s="206">
+      <c r="A29" s="239">
+        <f>IF(C29="","",$C$2&amp;"."&amp;COUNTA($C$8:C29)&amp;"")</f>
         <v/>
       </c>
-      <c r="B28" s="239" t="inlineStr">
-        <is>
-          <t>REQ-ASN-003</t>
-        </is>
-      </c>
-      <c r="C28" s="239" t="inlineStr">
-        <is>
-          <t>DOC-v1.0-01 §A5 (BR-CON-02)</t>
-        </is>
-      </c>
-      <c r="D28" s="239" t="inlineStr">
+      <c r="B29" s="239" t="inlineStr">
+        <is>
+          <t>REQ-ORD-001, REQ-ASN-002</t>
+        </is>
+      </c>
+      <c r="C29" s="239" t="inlineStr">
+        <is>
+          <t>DOC-v1.0-02 §3.4 Table 5</t>
+        </is>
+      </c>
+      <c r="D29" s="239" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="E28" s="239" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F28" s="239" t="inlineStr">
-        <is>
-          <t>Check SĐT người gửi KHÔNG hiển thị tại Chi tiết tin khi tin còn "Chờ ghép"</t>
-        </is>
-      </c>
-      <c r="G28" s="239" t="inlineStr">
-        <is>
-          <t>Tin đang ở trạng thái "Chờ ghép", chưa có ai xác nhận mang giúp; người xem là Carrier khác (không phải chủ tin)</t>
-        </is>
-      </c>
-      <c r="H28" s="239" t="inlineStr">
+      <c r="E29" s="239" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F29" s="239" t="inlineStr">
+        <is>
+          <t>Check đầy đủ + đúng 4 nhóm thông tin tại block "Lộ trình &amp; liên hệ" màn Chi tiết tin</t>
+        </is>
+      </c>
+      <c r="G29" s="239" t="inlineStr">
+        <is>
+          <t>Tin đang ở trạng thái "Chờ ghép", người xem là Carrier (không phải chủ tin)</t>
+        </is>
+      </c>
+      <c r="H29" s="239" t="inlineStr">
         <is>
           <t>1. Mở app FoxEco
 2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
-3. Quan sát phần thông tin "Người gửi" trong block "Lộ trình &amp; liên hệ"</t>
-        </is>
-      </c>
-      <c r="I28" s="239" t="inlineStr">
-        <is>
-          <t>3. SĐT của Người gửi KHÔNG hiển thị (chỉ hiện Tên) và nút "Gọi" không khả dụng</t>
-        </is>
-      </c>
-      <c r="J28" s="239" t="inlineStr">
+3. Quan sát block "Lộ trình &amp; liên hệ"</t>
+        </is>
+      </c>
+      <c r="I29" s="239" t="inlineStr">
+        <is>
+          <t>3. Block hiển thị đủ 4 nhóm: (1) Lộ trình gồm điểm Lấy hàng + điểm Giao hàng + khung "Bản đồ · ~X km", (2) Khung giờ mong muốn giao nhận, (3) Người gửi — hiển thị Tên (SĐT và nút "Gọi" CHƯA khả dụng khi tin còn "Chờ ghép", theo BR-CON-02/C-ASN-01), (4) nút "Tôi mang giúp được"</t>
+        </is>
+      </c>
+      <c r="J29" s="239" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="K28" s="239" t="inlineStr">
+      <c r="K29" s="239" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L28" s="239" t="inlineStr">
+      <c r="L29" s="239" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M28" s="239" t="n"/>
-      <c r="N28" s="239" t="n"/>
-      <c r="O28" s="239" t="n"/>
-      <c r="P28" s="239" t="n"/>
-      <c r="Q28" s="239" t="n"/>
-      <c r="R28" s="239" t="n"/>
-      <c r="S28" s="239" t="n"/>
-      <c r="T28" s="239" t="n"/>
-      <c r="U28" s="239" t="n"/>
-      <c r="V28" s="239" t="n"/>
-      <c r="W28" s="239" t="n"/>
-      <c r="X28" s="239" t="n"/>
-      <c r="Y28" s="239" t="n"/>
-      <c r="Z28" s="239" t="n"/>
-      <c r="AA28" s="239" t="n"/>
-      <c r="AB28" s="240" t="n"/>
-      <c r="AC28" s="240" t="n"/>
-      <c r="AD28" s="240" t="n"/>
-      <c r="AE28" s="240" t="n"/>
-      <c r="AF28" s="240" t="n"/>
-      <c r="AG28" s="240" t="n"/>
-      <c r="AH28" s="240" t="n"/>
-      <c r="AI28" s="240" t="n"/>
-      <c r="AJ28" s="240" t="n"/>
-      <c r="AK28" s="240" t="n"/>
-      <c r="AL28" s="240" t="n"/>
-      <c r="AM28" s="241">
-        <f>IF($A28="","",IF(OR($N28="Yes",$S28="Yes",$X28="Yes",$AC28="Yes",$AH28="Yes"),"Yes","No"))</f>
+      <c r="M29" s="239" t="n"/>
+      <c r="N29" s="239" t="n"/>
+      <c r="O29" s="239" t="n"/>
+      <c r="P29" s="239" t="n"/>
+      <c r="Q29" s="239" t="n"/>
+      <c r="R29" s="239" t="n"/>
+      <c r="S29" s="239" t="n"/>
+      <c r="T29" s="239" t="n"/>
+      <c r="U29" s="239" t="n"/>
+      <c r="V29" s="239" t="n"/>
+      <c r="W29" s="239" t="n"/>
+      <c r="X29" s="239" t="n"/>
+      <c r="Y29" s="239" t="n"/>
+      <c r="Z29" s="239" t="n"/>
+      <c r="AA29" s="239" t="n"/>
+      <c r="AB29" s="240" t="n"/>
+      <c r="AC29" s="240" t="n"/>
+      <c r="AD29" s="240" t="n"/>
+      <c r="AE29" s="240" t="n"/>
+      <c r="AF29" s="240" t="n"/>
+      <c r="AG29" s="240" t="n"/>
+      <c r="AH29" s="240" t="n"/>
+      <c r="AI29" s="240" t="n"/>
+      <c r="AJ29" s="240" t="n"/>
+      <c r="AK29" s="240" t="n"/>
+      <c r="AL29" s="240" t="n"/>
+      <c r="AM29" s="241">
+        <f>IF($A26="","",IF(OR($N26="Yes",$S26="Yes",$X26="Yes",$AC26="Yes",$AH26="Yes"),"Yes","No"))</f>
         <v/>
       </c>
-      <c r="AN28" s="241">
-        <f>IF($A28="","",IFERROR(IF($AI28&lt;&gt;"",$AI28,IF($AD28&lt;&gt;"",$AD28,IF($Y28&lt;&gt;"",$Y28,IF($T28&lt;&gt;"",$T28,IF($O28&lt;&gt;"",$O28,""))))),""))</f>
+      <c r="AN29" s="241">
+        <f>IF($A26="","",IFERROR(IF($AI26&lt;&gt;"",$AI26,IF($AD26&lt;&gt;"",$AD26,IF($Y26&lt;&gt;"",$Y26,IF($T26&lt;&gt;"",$T26,IF($O26&lt;&gt;"",$O26,""))))),""))</f>
         <v/>
       </c>
-      <c r="AO28" s="241">
-        <f>IFERROR(IF($AJ28&lt;&gt;"",$AJ28,IF($AE28&lt;&gt;"",$AE28,IF($Z28&lt;&gt;"",$Z28,IF($U28&lt;&gt;"",$U28,IF($P28&lt;&gt;"",$P28,""))))),"")</f>
+      <c r="AO29" s="241">
+        <f>IFERROR(IF($AJ26&lt;&gt;"",$AJ26,IF($AE26&lt;&gt;"",$AE26,IF($Z26&lt;&gt;"",$Z26,IF($U26&lt;&gt;"",$U26,IF($P26&lt;&gt;"",$P26,""))))),"")</f>
         <v/>
       </c>
-      <c r="AP28" s="240" t="inlineStr">
-        <is>
-          <t>Regression theo rule chính thức BR-CON-02 / C-ASN-01 (Resolved 2026-07-27) — bản demo hiện tại có thể lộ SĐT sớm (là BUG), TC này chủ đích bắt gap đó</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1" s="206">
-      <c r="A29" s="231" t="n"/>
-      <c r="B29" s="248" t="inlineStr">
-        <is>
-          <t>Block Chi tiết tin — Nút hành động vận chuyển</t>
-        </is>
-      </c>
-      <c r="C29" s="211" t="n"/>
-      <c r="D29" s="211" t="n"/>
-      <c r="E29" s="211" t="n"/>
-      <c r="F29" s="211" t="n"/>
-      <c r="G29" s="211" t="n"/>
-      <c r="H29" s="211" t="n"/>
-      <c r="I29" s="209" t="n"/>
-      <c r="J29" s="231" t="n"/>
-      <c r="K29" s="231" t="n"/>
-      <c r="L29" s="231" t="n"/>
-      <c r="M29" s="231" t="n"/>
-      <c r="N29" s="235" t="n"/>
-      <c r="O29" s="235" t="n"/>
-      <c r="P29" s="235" t="n"/>
-      <c r="Q29" s="235" t="n"/>
-      <c r="R29" s="235" t="n"/>
-      <c r="S29" s="235" t="n"/>
-      <c r="T29" s="235" t="n"/>
-      <c r="U29" s="235" t="n"/>
-      <c r="V29" s="235" t="n"/>
-      <c r="W29" s="235" t="n"/>
-      <c r="X29" s="235" t="n"/>
-      <c r="Y29" s="235" t="n"/>
-      <c r="Z29" s="235" t="n"/>
-      <c r="AA29" s="235" t="n"/>
-      <c r="AB29" s="236" t="n"/>
-      <c r="AC29" s="236" t="n"/>
-      <c r="AD29" s="236" t="n"/>
-      <c r="AE29" s="236" t="n"/>
-      <c r="AF29" s="236" t="n"/>
-      <c r="AG29" s="236" t="n"/>
-      <c r="AH29" s="236" t="n"/>
-      <c r="AI29" s="236" t="n"/>
-      <c r="AJ29" s="236" t="n"/>
-      <c r="AK29" s="236" t="n"/>
-      <c r="AL29" s="236" t="n"/>
-      <c r="AM29" s="237" t="n"/>
-      <c r="AN29" s="237" t="n"/>
-      <c r="AO29" s="237" t="n"/>
-      <c r="AP29" s="238" t="n"/>
+      <c r="AP29" s="240" t="inlineStr">
+        <is>
+          <t>Field/column completeness check — auto-derived (xem generate.md Step 3b) | Trường SĐT + nút "Gọi" chỉ khả dụng SAU khi ghép (BR-CON-02, C-ASN-01 Resolved) — xem TC regression SĐT không lộ + TC lộ SĐT sau ghép</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="60" customHeight="1" s="206">
       <c r="A30" s="239">
@@ -4721,44 +4784,44 @@
       </c>
       <c r="B30" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-001</t>
+          <t>REQ-ORD-001</t>
         </is>
       </c>
       <c r="C30" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §D3 (ASN-01) + DOC-v1.0-02 §4.2</t>
+          <t>DOC-v1.0-02 §3.4 Table 5</t>
         </is>
       </c>
       <c r="D30" s="239" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E30" s="239" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F30" s="239" t="inlineStr">
         <is>
-          <t>Check bấm "Tôi mang giúp được" khi tin còn "Chờ ghép" mở modal xác nhận</t>
+          <t>Check khung "Bản đồ · ~X km" hiển thị đúng dạng placeholder tĩnh</t>
         </is>
       </c>
       <c r="G30" s="239" t="inlineStr">
         <is>
-          <t>Tin đang ở "Chờ ghép"; người xem là Carrier, KHÔNG phải chủ tin và KHÔNG phải Người nhận của đơn</t>
+          <t>Tin đang ở trạng thái "Chờ ghép" với 2 địa chỉ lấy/giao khác nhau</t>
         </is>
       </c>
       <c r="H30" s="239" t="inlineStr">
         <is>
           <t>1. Mở app FoxEco
 2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
-3. Bấm nút "Tôi mang giúp được"</t>
+3. Quan sát khung bản đồ trong block "Lộ trình &amp; liên hệ" và thử bấm vào khung đó</t>
         </is>
       </c>
       <c r="I30" s="239" t="inlineStr">
         <is>
-          <t>3. Hiển thị modal "Xác nhận mang giúp"; đơn CHƯA đổi trạng thái (vẫn "Chờ ghép") cho tới khi bấm Xác nhận</t>
+          <t>3. Khung hiển thị đúng dạng text "Bản đồ · ~[N] km"; đây là placeholder tĩnh — bấm vào KHÔNG mở bản đồ thật, không phát sinh điều hướng</t>
         </is>
       </c>
       <c r="J30" s="239" t="inlineStr">
@@ -4803,15 +4866,15 @@
       <c r="AK30" s="240" t="n"/>
       <c r="AL30" s="240" t="n"/>
       <c r="AM30" s="241">
-        <f>IF($A30="","",IF(OR($N30="Yes",$S30="Yes",$X30="Yes",$AC30="Yes",$AH30="Yes"),"Yes","No"))</f>
+        <f>IF($A27="","",IF(OR($N27="Yes",$S27="Yes",$X27="Yes",$AC27="Yes",$AH27="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN30" s="241">
-        <f>IF($A30="","",IFERROR(IF($AI30&lt;&gt;"",$AI30,IF($AD30&lt;&gt;"",$AD30,IF($Y30&lt;&gt;"",$Y30,IF($T30&lt;&gt;"",$T30,IF($O30&lt;&gt;"",$O30,""))))),""))</f>
+        <f>IF($A27="","",IFERROR(IF($AI27&lt;&gt;"",$AI27,IF($AD27&lt;&gt;"",$AD27,IF($Y27&lt;&gt;"",$Y27,IF($T27&lt;&gt;"",$T27,IF($O27&lt;&gt;"",$O27,""))))),""))</f>
         <v/>
       </c>
       <c r="AO30" s="241">
-        <f>IFERROR(IF($AJ30&lt;&gt;"",$AJ30,IF($AE30&lt;&gt;"",$AE30,IF($Z30&lt;&gt;"",$Z30,IF($U30&lt;&gt;"",$U30,IF($P30&lt;&gt;"",$P30,""))))),"")</f>
+        <f>IFERROR(IF($AJ27&lt;&gt;"",$AJ27,IF($AE27&lt;&gt;"",$AE27,IF($Z27&lt;&gt;"",$Z27,IF($U27&lt;&gt;"",$U27,IF($P27&lt;&gt;"",$P27,""))))),"")</f>
         <v/>
       </c>
       <c r="AP30" s="240" t="n"/>
@@ -4823,44 +4886,44 @@
       </c>
       <c r="B31" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-001</t>
+          <t>REQ-ASN-003</t>
         </is>
       </c>
       <c r="C31" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §D3 (ASN-01) + DOC-v1.0-02 §4.2</t>
+          <t>DOC-v1.0-01 §A5 (BR-CON-02)</t>
         </is>
       </c>
       <c r="D31" s="239" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E31" s="239" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F31" s="239" t="inlineStr">
         <is>
-          <t>Check Sender nhận được thông báo push + in-app khi Carrier gửi đề nghị mang giúp</t>
+          <t>Check SĐT người gửi KHÔNG hiển thị tại Chi tiết tin khi tin còn "Chờ ghép"</t>
         </is>
       </c>
       <c r="G31" s="239" t="inlineStr">
         <is>
-          <t>Carrier vừa xác nhận mang giúp 1 tin của Sender; thiết bị của Sender đang bật thông báo</t>
+          <t>Tin đang ở trạng thái "Chờ ghép", chưa có ai xác nhận mang giúp; người xem là Carrier khác (không phải chủ tin)</t>
         </is>
       </c>
       <c r="H31" s="239" t="inlineStr">
         <is>
-          <t>1. Trên thiết bị Carrier: mở Chi tiết tin của tin "Chờ ghép", bấm "Tôi mang giúp được" rồi "Xác nhận"
-2. Chuyển sang thiết bị của Sender (chủ tin)
-3. Quan sát thông báo push và danh sách thông báo in-app</t>
+          <t>1. Mở app FoxEco
+2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
+3. Quan sát phần thông tin "Người gửi" trong block "Lộ trình &amp; liên hệ"</t>
         </is>
       </c>
       <c r="I31" s="239" t="inlineStr">
         <is>
-          <t>3. Sender nhận được cả thông báo push lẫn thông báo in-app về đề nghị mang giúp của Carrier đó</t>
+          <t>3. SĐT của Người gửi KHÔNG hiển thị (chỉ hiện Tên) và nút "Gọi" không khả dụng</t>
         </is>
       </c>
       <c r="J31" s="239" t="inlineStr">
@@ -4905,124 +4968,70 @@
       <c r="AK31" s="240" t="n"/>
       <c r="AL31" s="240" t="n"/>
       <c r="AM31" s="241">
-        <f>IF($A31="","",IF(OR($N31="Yes",$S31="Yes",$X31="Yes",$AC31="Yes",$AH31="Yes"),"Yes","No"))</f>
+        <f>IF($A28="","",IF(OR($N28="Yes",$S28="Yes",$X28="Yes",$AC28="Yes",$AH28="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN31" s="241">
-        <f>IF($A31="","",IFERROR(IF($AI31&lt;&gt;"",$AI31,IF($AD31&lt;&gt;"",$AD31,IF($Y31&lt;&gt;"",$Y31,IF($T31&lt;&gt;"",$T31,IF($O31&lt;&gt;"",$O31,""))))),""))</f>
+        <f>IF($A28="","",IFERROR(IF($AI28&lt;&gt;"",$AI28,IF($AD28&lt;&gt;"",$AD28,IF($Y28&lt;&gt;"",$Y28,IF($T28&lt;&gt;"",$T28,IF($O28&lt;&gt;"",$O28,""))))),""))</f>
         <v/>
       </c>
       <c r="AO31" s="241">
-        <f>IFERROR(IF($AJ31&lt;&gt;"",$AJ31,IF($AE31&lt;&gt;"",$AE31,IF($Z31&lt;&gt;"",$Z31,IF($U31&lt;&gt;"",$U31,IF($P31&lt;&gt;"",$P31,""))))),"")</f>
+        <f>IFERROR(IF($AJ28&lt;&gt;"",$AJ28,IF($AE28&lt;&gt;"",$AE28,IF($Z28&lt;&gt;"",$Z28,IF($U28&lt;&gt;"",$U28,IF($P28&lt;&gt;"",$P28,""))))),"")</f>
         <v/>
       </c>
-      <c r="AP31" s="240" t="n"/>
-    </row>
-    <row r="32" ht="60" customHeight="1" s="206">
-      <c r="A32" s="239">
-        <f>IF(C32="","",$C$2&amp;"."&amp;COUNTA($C$8:C32)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="B32" s="239" t="inlineStr">
-        <is>
-          <t>REQ-ASN-008</t>
-        </is>
-      </c>
-      <c r="C32" s="239" t="inlineStr">
-        <is>
-          <t>DOC-v1.0-01 §D7 (OPR-05) + DOC-v1.0-02 §3.3</t>
-        </is>
-      </c>
-      <c r="D32" s="239" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="E32" s="239" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F32" s="239" t="inlineStr">
-        <is>
-          <t>Check nút "Tôi mang giúp được" ẨN/disable khi người xem chính là chủ tin</t>
-        </is>
-      </c>
-      <c r="G32" s="239" t="inlineStr">
-        <is>
-          <t>Tin do chính user đang đăng nhập đăng (vai trò Sender), tin đang ở "Chờ ghép"</t>
-        </is>
-      </c>
-      <c r="H32" s="239" t="inlineStr">
-        <is>
-          <t>1. Mở app FoxEco bằng tài khoản đã đăng tin
-2. Bấm tab "Bảng tin", mở Chi tiết tin của chính tin mình đăng
-3. Quan sát vùng nút hành động vận chuyển</t>
-        </is>
-      </c>
-      <c r="I32" s="239" t="inlineStr">
-        <is>
-          <t>3. Nút "Tôi mang giúp được" bị ẩn hoặc disable — chủ tin KHÔNG tự nhận mang giúp tin của mình được</t>
-        </is>
-      </c>
-      <c r="J32" s="239" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="K32" s="239" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L32" s="239" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M32" s="239" t="n"/>
-      <c r="N32" s="239" t="n"/>
-      <c r="O32" s="239" t="n"/>
-      <c r="P32" s="239" t="n"/>
-      <c r="Q32" s="239" t="n"/>
-      <c r="R32" s="239" t="n"/>
-      <c r="S32" s="239" t="n"/>
-      <c r="T32" s="239" t="n"/>
-      <c r="U32" s="239" t="n"/>
-      <c r="V32" s="239" t="n"/>
-      <c r="W32" s="239" t="n"/>
-      <c r="X32" s="239" t="n"/>
-      <c r="Y32" s="239" t="n"/>
-      <c r="Z32" s="239" t="n"/>
-      <c r="AA32" s="239" t="n"/>
-      <c r="AB32" s="240" t="n"/>
-      <c r="AC32" s="240" t="n"/>
-      <c r="AD32" s="240" t="n"/>
-      <c r="AE32" s="240" t="n"/>
-      <c r="AF32" s="240" t="n"/>
-      <c r="AG32" s="240" t="n"/>
-      <c r="AH32" s="240" t="n"/>
-      <c r="AI32" s="240" t="n"/>
-      <c r="AJ32" s="240" t="n"/>
-      <c r="AK32" s="240" t="n"/>
-      <c r="AL32" s="240" t="n"/>
-      <c r="AM32" s="241">
-        <f>IF($A32="","",IF(OR($N32="Yes",$S32="Yes",$X32="Yes",$AC32="Yes",$AH32="Yes"),"Yes","No"))</f>
-        <v/>
-      </c>
-      <c r="AN32" s="241">
-        <f>IF($A32="","",IFERROR(IF($AI32&lt;&gt;"",$AI32,IF($AD32&lt;&gt;"",$AD32,IF($Y32&lt;&gt;"",$Y32,IF($T32&lt;&gt;"",$T32,IF($O32&lt;&gt;"",$O32,""))))),""))</f>
-        <v/>
-      </c>
-      <c r="AO32" s="241">
-        <f>IFERROR(IF($AJ32&lt;&gt;"",$AJ32,IF($AE32&lt;&gt;"",$AE32,IF($Z32&lt;&gt;"",$Z32,IF($U32&lt;&gt;"",$U32,IF($P32&lt;&gt;"",$P32,""))))),"")</f>
-        <v/>
-      </c>
-      <c r="AP32" s="240" t="inlineStr">
-        <is>
-          <t>Technique: EP-viewer-owner | Regression theo OPR-05 / C-ASN-02 (Resolved 2026-07-27) — bản demo hiện tại vi phạm rule này (DOC-v1.0-02 §3.3 Lưu ý ⚠), TC chủ đích bắt gap</t>
-        </is>
-      </c>
+      <c r="AP31" s="240" t="inlineStr">
+        <is>
+          <t>Regression theo rule chính thức BR-CON-02 / C-ASN-01 (Resolved 2026-07-27) — bản demo hiện tại có thể lộ SĐT sớm (là BUG), TC này chủ đích bắt gap đó</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1" s="206">
+      <c r="A32" s="231" t="n"/>
+      <c r="B32" s="248" t="inlineStr">
+        <is>
+          <t>Block Chi tiết tin — Nút hành động vận chuyển</t>
+        </is>
+      </c>
+      <c r="C32" s="211" t="n"/>
+      <c r="D32" s="211" t="n"/>
+      <c r="E32" s="211" t="n"/>
+      <c r="F32" s="211" t="n"/>
+      <c r="G32" s="211" t="n"/>
+      <c r="H32" s="211" t="n"/>
+      <c r="I32" s="209" t="n"/>
+      <c r="J32" s="231" t="n"/>
+      <c r="K32" s="231" t="n"/>
+      <c r="L32" s="231" t="n"/>
+      <c r="M32" s="231" t="n"/>
+      <c r="N32" s="235" t="n"/>
+      <c r="O32" s="235" t="n"/>
+      <c r="P32" s="235" t="n"/>
+      <c r="Q32" s="235" t="n"/>
+      <c r="R32" s="235" t="n"/>
+      <c r="S32" s="235" t="n"/>
+      <c r="T32" s="235" t="n"/>
+      <c r="U32" s="235" t="n"/>
+      <c r="V32" s="235" t="n"/>
+      <c r="W32" s="235" t="n"/>
+      <c r="X32" s="235" t="n"/>
+      <c r="Y32" s="235" t="n"/>
+      <c r="Z32" s="235" t="n"/>
+      <c r="AA32" s="235" t="n"/>
+      <c r="AB32" s="236" t="n"/>
+      <c r="AC32" s="236" t="n"/>
+      <c r="AD32" s="236" t="n"/>
+      <c r="AE32" s="236" t="n"/>
+      <c r="AF32" s="236" t="n"/>
+      <c r="AG32" s="236" t="n"/>
+      <c r="AH32" s="236" t="n"/>
+      <c r="AI32" s="236" t="n"/>
+      <c r="AJ32" s="236" t="n"/>
+      <c r="AK32" s="236" t="n"/>
+      <c r="AL32" s="236" t="n"/>
+      <c r="AM32" s="237" t="n"/>
+      <c r="AN32" s="237" t="n"/>
+      <c r="AO32" s="237" t="n"/>
+      <c r="AP32" s="238" t="n"/>
     </row>
     <row r="33" ht="60" customHeight="1" s="206">
       <c r="A33" s="239">
@@ -5031,17 +5040,17 @@
       </c>
       <c r="B33" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-008</t>
+          <t>REQ-ASN-001</t>
         </is>
       </c>
       <c r="C33" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §D7 (OPR-05) + DOC-v1.0-02 §3.3</t>
+          <t>DOC-v1.0-01 §D3 (ASN-01) + DOC-v1.0-02 §4.2</t>
         </is>
       </c>
       <c r="D33" s="239" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="E33" s="239" t="inlineStr">
@@ -5051,24 +5060,24 @@
       </c>
       <c r="F33" s="239" t="inlineStr">
         <is>
-          <t>Check nút "Tôi mang giúp được" ẨN/disable khi người xem là Người nhận của đơn</t>
+          <t>Check bấm "Tôi mang giúp được" khi tin còn "Chờ ghép" mở modal xác nhận</t>
         </is>
       </c>
       <c r="G33" s="239" t="inlineStr">
         <is>
-          <t>Tin đang ở "Chờ ghép"; user đang đăng nhập là Người nhận (Receiver) được khai báo trên chính tin đó</t>
+          <t>Tin đang ở "Chờ ghép"; người xem là Carrier, KHÔNG phải chủ tin và KHÔNG phải Người nhận của đơn</t>
         </is>
       </c>
       <c r="H33" s="239" t="inlineStr">
         <is>
-          <t>1. Mở app FoxEco bằng tài khoản là Người nhận của tin
-2. Bấm tab "Bảng tin", mở Chi tiết tin của tin đó
-3. Quan sát vùng nút hành động vận chuyển</t>
+          <t>1. Mở app FoxEco
+2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
+3. Bấm nút "Tôi mang giúp được"</t>
         </is>
       </c>
       <c r="I33" s="239" t="inlineStr">
         <is>
-          <t>3. Nút "Tôi mang giúp được" bị ẩn hoặc disable — Người nhận KHÔNG đồng thời làm người vận chuyển của cùng đơn</t>
+          <t>3. Hiển thị modal "Xác nhận mang giúp"; đơn CHƯA đổi trạng thái (vẫn "Chờ ghép") cho tới khi bấm Xác nhận</t>
         </is>
       </c>
       <c r="J33" s="239" t="inlineStr">
@@ -5113,22 +5122,18 @@
       <c r="AK33" s="240" t="n"/>
       <c r="AL33" s="240" t="n"/>
       <c r="AM33" s="241">
-        <f>IF($A33="","",IF(OR($N33="Yes",$S33="Yes",$X33="Yes",$AC33="Yes",$AH33="Yes"),"Yes","No"))</f>
+        <f>IF($A30="","",IF(OR($N30="Yes",$S30="Yes",$X30="Yes",$AC30="Yes",$AH30="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN33" s="241">
-        <f>IF($A33="","",IFERROR(IF($AI33&lt;&gt;"",$AI33,IF($AD33&lt;&gt;"",$AD33,IF($Y33&lt;&gt;"",$Y33,IF($T33&lt;&gt;"",$T33,IF($O33&lt;&gt;"",$O33,""))))),""))</f>
+        <f>IF($A30="","",IFERROR(IF($AI30&lt;&gt;"",$AI30,IF($AD30&lt;&gt;"",$AD30,IF($Y30&lt;&gt;"",$Y30,IF($T30&lt;&gt;"",$T30,IF($O30&lt;&gt;"",$O30,""))))),""))</f>
         <v/>
       </c>
       <c r="AO33" s="241">
-        <f>IFERROR(IF($AJ33&lt;&gt;"",$AJ33,IF($AE33&lt;&gt;"",$AE33,IF($Z33&lt;&gt;"",$Z33,IF($U33&lt;&gt;"",$U33,IF($P33&lt;&gt;"",$P33,""))))),"")</f>
+        <f>IFERROR(IF($AJ30&lt;&gt;"",$AJ30,IF($AE30&lt;&gt;"",$AE30,IF($Z30&lt;&gt;"",$Z30,IF($U30&lt;&gt;"",$U30,IF($P30&lt;&gt;"",$P30,""))))),"")</f>
         <v/>
       </c>
-      <c r="AP33" s="240" t="inlineStr">
-        <is>
-          <t>Technique: EP-viewer-receiver | Regression theo OPR-05 / C-ASN-02 (Resolved 2026-07-27)</t>
-        </is>
-      </c>
+      <c r="AP33" s="240" t="n"/>
     </row>
     <row r="34" ht="60" customHeight="1" s="206">
       <c r="A34" s="239">
@@ -5137,17 +5142,17 @@
       </c>
       <c r="B34" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-008</t>
+          <t>REQ-ASN-001</t>
         </is>
       </c>
       <c r="C34" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §D7 (OPR-05) + DOC-v1.0-02 §3.3</t>
+          <t>DOC-v1.0-01 §D3 (ASN-01) + DOC-v1.0-02 §4.2</t>
         </is>
       </c>
       <c r="D34" s="239" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="E34" s="239" t="inlineStr">
@@ -5157,24 +5162,24 @@
       </c>
       <c r="F34" s="239" t="inlineStr">
         <is>
-          <t>Check nút "Tôi mang giúp được" HIỂN THỊ khi người xem là bên thứ ba</t>
+          <t>Check Sender nhận được thông báo push + in-app khi Carrier gửi đề nghị mang giúp</t>
         </is>
       </c>
       <c r="G34" s="239" t="inlineStr">
         <is>
-          <t>Tin đang ở "Chờ ghép"; user đang đăng nhập KHÔNG phải chủ tin và KHÔNG phải Người nhận của đơn</t>
+          <t>Carrier vừa xác nhận mang giúp 1 tin của Sender; thiết bị của Sender đang bật thông báo</t>
         </is>
       </c>
       <c r="H34" s="239" t="inlineStr">
         <is>
-          <t>1. Mở app FoxEco
-2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
-3. Quan sát vùng nút hành động vận chuyển</t>
+          <t>1. Trên thiết bị Carrier: mở Chi tiết tin của tin "Chờ ghép", bấm "Tôi mang giúp được" rồi "Xác nhận"
+2. Chuyển sang thiết bị của Sender (chủ tin)
+3. Quan sát thông báo push và danh sách thông báo in-app</t>
         </is>
       </c>
       <c r="I34" s="239" t="inlineStr">
         <is>
-          <t>3. Nút "Tôi mang giúp được" hiển thị bình thường và bấm được</t>
+          <t>3. Sender nhận được cả thông báo push lẫn thông báo in-app về đề nghị mang giúp của Carrier đó</t>
         </is>
       </c>
       <c r="J34" s="239" t="inlineStr">
@@ -5219,22 +5224,18 @@
       <c r="AK34" s="240" t="n"/>
       <c r="AL34" s="240" t="n"/>
       <c r="AM34" s="241">
-        <f>IF($A34="","",IF(OR($N34="Yes",$S34="Yes",$X34="Yes",$AC34="Yes",$AH34="Yes"),"Yes","No"))</f>
+        <f>IF($A31="","",IF(OR($N31="Yes",$S31="Yes",$X31="Yes",$AC31="Yes",$AH31="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN34" s="241">
-        <f>IF($A34="","",IFERROR(IF($AI34&lt;&gt;"",$AI34,IF($AD34&lt;&gt;"",$AD34,IF($Y34&lt;&gt;"",$Y34,IF($T34&lt;&gt;"",$T34,IF($O34&lt;&gt;"",$O34,""))))),""))</f>
+        <f>IF($A31="","",IFERROR(IF($AI31&lt;&gt;"",$AI31,IF($AD31&lt;&gt;"",$AD31,IF($Y31&lt;&gt;"",$Y31,IF($T31&lt;&gt;"",$T31,IF($O31&lt;&gt;"",$O31,""))))),""))</f>
         <v/>
       </c>
       <c r="AO34" s="241">
-        <f>IFERROR(IF($AJ34&lt;&gt;"",$AJ34,IF($AE34&lt;&gt;"",$AE34,IF($Z34&lt;&gt;"",$Z34,IF($U34&lt;&gt;"",$U34,IF($P34&lt;&gt;"",$P34,""))))),"")</f>
+        <f>IFERROR(IF($AJ31&lt;&gt;"",$AJ31,IF($AE31&lt;&gt;"",$AE31,IF($Z31&lt;&gt;"",$Z31,IF($U31&lt;&gt;"",$U31,IF($P31&lt;&gt;"",$P31,""))))),"")</f>
         <v/>
       </c>
-      <c r="AP34" s="240" t="inlineStr">
-        <is>
-          <t>Technique: EP-viewer-third-party (partition hợp lệ, đối chứng cho 2 partition bị cấm ở trên)</t>
-        </is>
-      </c>
+      <c r="AP34" s="240" t="n"/>
     </row>
     <row r="35" ht="60" customHeight="1" s="206">
       <c r="A35" s="239">
@@ -5258,29 +5259,29 @@
       </c>
       <c r="E35" s="239" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F35" s="239" t="inlineStr">
         <is>
-          <t>Check tin do chính user đăng VẪN hiển thị bình thường trong danh sách Bảng tin</t>
+          <t>Check nút "Tôi mang giúp được" ẨN/disable khi người xem chính là chủ tin</t>
         </is>
       </c>
       <c r="G35" s="239" t="inlineStr">
         <is>
-          <t>User đã đăng ít nhất 1 tin đang ở trạng thái "Chờ ghép"</t>
+          <t>Tin do chính user đang đăng nhập đăng (vai trò Sender), tin đang ở "Chờ ghép"</t>
         </is>
       </c>
       <c r="H35" s="239" t="inlineStr">
         <is>
-          <t>1. Mở app FoxEco
-2. Bấm tab "Bảng tin" tại bottom nav
-3. Tìm tin do chính user đăng trong danh sách</t>
+          <t>1. Mở app FoxEco bằng tài khoản đã đăng tin
+2. Bấm tab "Bảng tin", mở Chi tiết tin của chính tin mình đăng
+3. Quan sát vùng nút hành động vận chuyển</t>
         </is>
       </c>
       <c r="I35" s="239" t="inlineStr">
         <is>
-          <t>3. Tin do chính user đăng VẪN xuất hiện trong danh sách Bảng tin (chỉ nút "Tôi mang giúp được" ở Chi tiết tin bị ẩn/disable, tin KHÔNG bị ẩn khỏi feed)</t>
+          <t>3. Nút "Tôi mang giúp được" bị ẩn hoặc disable — chủ tin KHÔNG tự nhận mang giúp tin của mình được</t>
         </is>
       </c>
       <c r="J35" s="239" t="inlineStr">
@@ -5325,20 +5326,20 @@
       <c r="AK35" s="240" t="n"/>
       <c r="AL35" s="240" t="n"/>
       <c r="AM35" s="241">
-        <f>IF($A35="","",IF(OR($N35="Yes",$S35="Yes",$X35="Yes",$AC35="Yes",$AH35="Yes"),"Yes","No"))</f>
+        <f>IF($A32="","",IF(OR($N32="Yes",$S32="Yes",$X32="Yes",$AC32="Yes",$AH32="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN35" s="241">
-        <f>IF($A35="","",IFERROR(IF($AI35&lt;&gt;"",$AI35,IF($AD35&lt;&gt;"",$AD35,IF($Y35&lt;&gt;"",$Y35,IF($T35&lt;&gt;"",$T35,IF($O35&lt;&gt;"",$O35,""))))),""))</f>
+        <f>IF($A32="","",IFERROR(IF($AI32&lt;&gt;"",$AI32,IF($AD32&lt;&gt;"",$AD32,IF($Y32&lt;&gt;"",$Y32,IF($T32&lt;&gt;"",$T32,IF($O32&lt;&gt;"",$O32,""))))),""))</f>
         <v/>
       </c>
       <c r="AO35" s="241">
-        <f>IFERROR(IF($AJ35&lt;&gt;"",$AJ35,IF($AE35&lt;&gt;"",$AE35,IF($Z35&lt;&gt;"",$Z35,IF($U35&lt;&gt;"",$U35,IF($P35&lt;&gt;"",$P35,""))))),"")</f>
+        <f>IFERROR(IF($AJ32&lt;&gt;"",$AJ32,IF($AE32&lt;&gt;"",$AE32,IF($Z32&lt;&gt;"",$Z32,IF($U32&lt;&gt;"",$U32,IF($P32&lt;&gt;"",$P32,""))))),"")</f>
         <v/>
       </c>
       <c r="AP35" s="240" t="inlineStr">
         <is>
-          <t>Đối chứng phân biệt phạm vi OPR-05: cấm ở tầng NÚT HÀNH ĐỘNG, không phải ẩn tin khỏi danh sách (xem Analyst Note Block "Danh sách tin đăng", test_scenario_map.md)</t>
+          <t>Technique: EP-viewer-owner | Regression theo OPR-05 / C-ASN-02 (Resolved 2026-07-27) — bản demo hiện tại vi phạm rule này (DOC-v1.0-02 §3.3 Lưu ý ⚠), TC chủ đích bắt gap</t>
         </is>
       </c>
     </row>
@@ -5349,44 +5350,44 @@
       </c>
       <c r="B36" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-004</t>
+          <t>REQ-ASN-008</t>
         </is>
       </c>
       <c r="C36" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §D3/§D4 (MTCH-01, BR-MTCH-01)</t>
+          <t>DOC-v1.0-01 §D7 (OPR-05) + DOC-v1.0-02 §3.3</t>
         </is>
       </c>
       <c r="D36" s="239" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E36" s="239" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F36" s="239" t="inlineStr">
         <is>
-          <t>Check Carrier bấm "Nhận giao" từ thông báo khớp tuyến → đơn chuyển "Đã ghép"</t>
+          <t>Check nút "Tôi mang giúp được" ẨN/disable khi người xem là Người nhận của đơn</t>
         </is>
       </c>
       <c r="G36" s="239" t="inlineStr">
         <is>
-          <t>Carrier đã đăng tuyến OFFER và vừa nhận thông báo khớp tuyến về 1 tin NEED phù hợp</t>
+          <t>Tin đang ở "Chờ ghép"; user đang đăng nhập là Người nhận (Receiver) được khai báo trên chính tin đó</t>
         </is>
       </c>
       <c r="H36" s="239" t="inlineStr">
         <is>
-          <t>1. Mở app FoxEco bằng tài khoản Carrier, mở màn Thông báo
-2. Bấm thông báo khớp tuyến để mở Chi tiết tin của tin NEED phù hợp
-3. Bấm "Nhận giao" và xác nhận</t>
+          <t>1. Mở app FoxEco bằng tài khoản là Người nhận của tin
+2. Bấm tab "Bảng tin", mở Chi tiết tin của tin đó
+3. Quan sát vùng nút hành động vận chuyển</t>
         </is>
       </c>
       <c r="I36" s="239" t="inlineStr">
         <is>
-          <t>3. Đơn chuyển sang trạng thái "Đã ghép", liên hệ 2 bên được lộ và Carrier vào được màn Theo dõi đơn</t>
+          <t>3. Nút "Tôi mang giúp được" bị ẩn hoặc disable — Người nhận KHÔNG đồng thời làm người vận chuyển của cùng đơn</t>
         </is>
       </c>
       <c r="J36" s="239" t="inlineStr">
@@ -5431,70 +5432,128 @@
       <c r="AK36" s="240" t="n"/>
       <c r="AL36" s="240" t="n"/>
       <c r="AM36" s="241">
-        <f>IF($A36="","",IF(OR($N36="Yes",$S36="Yes",$X36="Yes",$AC36="Yes",$AH36="Yes"),"Yes","No"))</f>
+        <f>IF($A33="","",IF(OR($N33="Yes",$S33="Yes",$X33="Yes",$AC33="Yes",$AH33="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN36" s="241">
-        <f>IF($A36="","",IFERROR(IF($AI36&lt;&gt;"",$AI36,IF($AD36&lt;&gt;"",$AD36,IF($Y36&lt;&gt;"",$Y36,IF($T36&lt;&gt;"",$T36,IF($O36&lt;&gt;"",$O36,""))))),""))</f>
+        <f>IF($A33="","",IFERROR(IF($AI33&lt;&gt;"",$AI33,IF($AD33&lt;&gt;"",$AD33,IF($Y33&lt;&gt;"",$Y33,IF($T33&lt;&gt;"",$T33,IF($O33&lt;&gt;"",$O33,""))))),""))</f>
         <v/>
       </c>
       <c r="AO36" s="241">
-        <f>IFERROR(IF($AJ36&lt;&gt;"",$AJ36,IF($AE36&lt;&gt;"",$AE36,IF($Z36&lt;&gt;"",$Z36,IF($U36&lt;&gt;"",$U36,IF($P36&lt;&gt;"",$P36,""))))),"")</f>
+        <f>IFERROR(IF($AJ33&lt;&gt;"",$AJ33,IF($AE33&lt;&gt;"",$AE33,IF($Z33&lt;&gt;"",$Z33,IF($U33&lt;&gt;"",$U33,IF($P33&lt;&gt;"",$P33,""))))),"")</f>
         <v/>
       </c>
       <c r="AP36" s="240" t="inlineStr">
         <is>
-          <t>⚠ Thuộc nhánh auto-match tuyến OFFER↔NEED — `Project_rule.md` Phase 1 Scope liệt kê nhánh này là NGOÀI phạm vi Phase 1 (PM chưa trả lời dứt điểm). Giữ TC để không mất coverage `SC-ASN-007`, đánh dấu chờ PM chốt scope trước khi đưa vào vòng chạy</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1" s="206">
-      <c r="A37" s="231" t="n"/>
-      <c r="B37" s="232" t="inlineStr">
-        <is>
-          <t>Block Modal xác nhận mang giúp</t>
-        </is>
-      </c>
-      <c r="C37" s="211" t="n"/>
-      <c r="D37" s="211" t="n"/>
-      <c r="E37" s="211" t="n"/>
-      <c r="F37" s="211" t="n"/>
-      <c r="G37" s="211" t="n"/>
-      <c r="H37" s="211" t="n"/>
-      <c r="I37" s="209" t="n"/>
-      <c r="J37" s="231" t="n"/>
-      <c r="K37" s="231" t="n"/>
-      <c r="L37" s="231" t="n"/>
-      <c r="M37" s="231" t="n"/>
-      <c r="N37" s="235" t="n"/>
-      <c r="O37" s="235" t="n"/>
-      <c r="P37" s="235" t="n"/>
-      <c r="Q37" s="235" t="n"/>
-      <c r="R37" s="235" t="n"/>
-      <c r="S37" s="235" t="n"/>
-      <c r="T37" s="235" t="n"/>
-      <c r="U37" s="235" t="n"/>
-      <c r="V37" s="235" t="n"/>
-      <c r="W37" s="235" t="n"/>
-      <c r="X37" s="235" t="n"/>
-      <c r="Y37" s="235" t="n"/>
-      <c r="Z37" s="235" t="n"/>
-      <c r="AA37" s="235" t="n"/>
-      <c r="AB37" s="236" t="n"/>
-      <c r="AC37" s="236" t="n"/>
-      <c r="AD37" s="236" t="n"/>
-      <c r="AE37" s="236" t="n"/>
-      <c r="AF37" s="236" t="n"/>
-      <c r="AG37" s="236" t="n"/>
-      <c r="AH37" s="236" t="n"/>
-      <c r="AI37" s="236" t="n"/>
-      <c r="AJ37" s="236" t="n"/>
-      <c r="AK37" s="236" t="n"/>
-      <c r="AL37" s="236" t="n"/>
-      <c r="AM37" s="237" t="n"/>
-      <c r="AN37" s="237" t="n"/>
-      <c r="AO37" s="237" t="n"/>
-      <c r="AP37" s="238" t="n"/>
+          <t>Technique: EP-viewer-receiver | Regression theo OPR-05 / C-ASN-02 (Resolved 2026-07-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="60" customHeight="1" s="206">
+      <c r="A37" s="239">
+        <f>IF(C37="","",$C$2&amp;"."&amp;COUNTA($C$8:C37)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="B37" s="239" t="inlineStr">
+        <is>
+          <t>REQ-ASN-008</t>
+        </is>
+      </c>
+      <c r="C37" s="239" t="inlineStr">
+        <is>
+          <t>DOC-v1.0-01 §D7 (OPR-05) + DOC-v1.0-02 §3.3</t>
+        </is>
+      </c>
+      <c r="D37" s="239" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E37" s="239" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F37" s="239" t="inlineStr">
+        <is>
+          <t>Check nút "Tôi mang giúp được" HIỂN THỊ khi người xem là bên thứ ba</t>
+        </is>
+      </c>
+      <c r="G37" s="239" t="inlineStr">
+        <is>
+          <t>Tin đang ở "Chờ ghép"; user đang đăng nhập KHÔNG phải chủ tin và KHÔNG phải Người nhận của đơn</t>
+        </is>
+      </c>
+      <c r="H37" s="239" t="inlineStr">
+        <is>
+          <t>1. Mở app FoxEco
+2. Bấm tab "Bảng tin", bấm vào 1 tin để mở màn Chi tiết tin
+3. Quan sát vùng nút hành động vận chuyển</t>
+        </is>
+      </c>
+      <c r="I37" s="239" t="inlineStr">
+        <is>
+          <t>3. Nút "Tôi mang giúp được" hiển thị bình thường và bấm được</t>
+        </is>
+      </c>
+      <c r="J37" s="239" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="K37" s="239" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L37" s="239" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M37" s="239" t="n"/>
+      <c r="N37" s="239" t="n"/>
+      <c r="O37" s="239" t="n"/>
+      <c r="P37" s="239" t="n"/>
+      <c r="Q37" s="239" t="n"/>
+      <c r="R37" s="239" t="n"/>
+      <c r="S37" s="239" t="n"/>
+      <c r="T37" s="239" t="n"/>
+      <c r="U37" s="239" t="n"/>
+      <c r="V37" s="239" t="n"/>
+      <c r="W37" s="239" t="n"/>
+      <c r="X37" s="239" t="n"/>
+      <c r="Y37" s="239" t="n"/>
+      <c r="Z37" s="239" t="n"/>
+      <c r="AA37" s="239" t="n"/>
+      <c r="AB37" s="240" t="n"/>
+      <c r="AC37" s="240" t="n"/>
+      <c r="AD37" s="240" t="n"/>
+      <c r="AE37" s="240" t="n"/>
+      <c r="AF37" s="240" t="n"/>
+      <c r="AG37" s="240" t="n"/>
+      <c r="AH37" s="240" t="n"/>
+      <c r="AI37" s="240" t="n"/>
+      <c r="AJ37" s="240" t="n"/>
+      <c r="AK37" s="240" t="n"/>
+      <c r="AL37" s="240" t="n"/>
+      <c r="AM37" s="241">
+        <f>IF($A34="","",IF(OR($N34="Yes",$S34="Yes",$X34="Yes",$AC34="Yes",$AH34="Yes"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="AN37" s="241">
+        <f>IF($A34="","",IFERROR(IF($AI34&lt;&gt;"",$AI34,IF($AD34&lt;&gt;"",$AD34,IF($Y34&lt;&gt;"",$Y34,IF($T34&lt;&gt;"",$T34,IF($O34&lt;&gt;"",$O34,""))))),""))</f>
+        <v/>
+      </c>
+      <c r="AO37" s="241">
+        <f>IFERROR(IF($AJ34&lt;&gt;"",$AJ34,IF($AE34&lt;&gt;"",$AE34,IF($Z34&lt;&gt;"",$Z34,IF($U34&lt;&gt;"",$U34,IF($P34&lt;&gt;"",$P34,""))))),"")</f>
+        <v/>
+      </c>
+      <c r="AP37" s="240" t="inlineStr">
+        <is>
+          <t>Technique: EP-viewer-third-party (partition hợp lệ, đối chứng cho 2 partition bị cấm ở trên)</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="60" customHeight="1" s="206">
       <c r="A38" s="239">
@@ -5503,12 +5562,12 @@
       </c>
       <c r="B38" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-002</t>
+          <t>REQ-ASN-008</t>
         </is>
       </c>
       <c r="C38" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §A5 (BR-CON-01/02) + DOC-v1.0-02 §4.2</t>
+          <t>DOC-v1.0-01 §D7 (OPR-05) + DOC-v1.0-02 §3.3</t>
         </is>
       </c>
       <c r="D38" s="239" t="inlineStr">
@@ -5523,24 +5582,24 @@
       </c>
       <c r="F38" s="239" t="inlineStr">
         <is>
-          <t>Check đầy đủ + đúng 3 thành phần hiển thị tại modal "Xác nhận mang giúp"</t>
+          <t>Check tin do chính user đăng VẪN hiển thị bình thường trong danh sách Bảng tin</t>
         </is>
       </c>
       <c r="G38" s="239" t="inlineStr">
         <is>
-          <t>Đang ở Chi tiết tin của 1 tin "Chờ ghép", đã bấm nút "Tôi mang giúp được"</t>
+          <t>User đã đăng ít nhất 1 tin đang ở trạng thái "Chờ ghép"</t>
         </is>
       </c>
       <c r="H38" s="239" t="inlineStr">
         <is>
           <t>1. Mở app FoxEco
-2. Bấm tab "Bảng tin", mở Chi tiết tin của 1 tin "Chờ ghép"
-3. Bấm "Tôi mang giúp được" và quan sát modal vừa hiện</t>
+2. Bấm tab "Bảng tin" tại bottom nav
+3. Tìm tin do chính user đăng trong danh sách</t>
         </is>
       </c>
       <c r="I38" s="239" t="inlineStr">
         <is>
-          <t>3. Modal hiển thị đủ 3 thành phần: (1) nội dung cảnh báo SĐT hai bên sẽ được lộ sau khi xác nhận, (2) nút "Huỷ", (3) nút "Xác nhận"</t>
+          <t>3. Tin do chính user đăng VẪN xuất hiện trong danh sách Bảng tin (chỉ nút "Tôi mang giúp được" ở Chi tiết tin bị ẩn/disable, tin KHÔNG bị ẩn khỏi feed)</t>
         </is>
       </c>
       <c r="J38" s="239" t="inlineStr">
@@ -5585,20 +5644,20 @@
       <c r="AK38" s="240" t="n"/>
       <c r="AL38" s="240" t="n"/>
       <c r="AM38" s="241">
-        <f>IF($A38="","",IF(OR($N38="Yes",$S38="Yes",$X38="Yes",$AC38="Yes",$AH38="Yes"),"Yes","No"))</f>
+        <f>IF($A35="","",IF(OR($N35="Yes",$S35="Yes",$X35="Yes",$AC35="Yes",$AH35="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN38" s="241">
-        <f>IF($A38="","",IFERROR(IF($AI38&lt;&gt;"",$AI38,IF($AD38&lt;&gt;"",$AD38,IF($Y38&lt;&gt;"",$Y38,IF($T38&lt;&gt;"",$T38,IF($O38&lt;&gt;"",$O38,""))))),""))</f>
+        <f>IF($A35="","",IFERROR(IF($AI35&lt;&gt;"",$AI35,IF($AD35&lt;&gt;"",$AD35,IF($Y35&lt;&gt;"",$Y35,IF($T35&lt;&gt;"",$T35,IF($O35&lt;&gt;"",$O35,""))))),""))</f>
         <v/>
       </c>
       <c r="AO38" s="241">
-        <f>IFERROR(IF($AJ38&lt;&gt;"",$AJ38,IF($AE38&lt;&gt;"",$AE38,IF($Z38&lt;&gt;"",$Z38,IF($U38&lt;&gt;"",$U38,IF($P38&lt;&gt;"",$P38,""))))),"")</f>
+        <f>IFERROR(IF($AJ35&lt;&gt;"",$AJ35,IF($AE35&lt;&gt;"",$AE35,IF($Z35&lt;&gt;"",$Z35,IF($U35&lt;&gt;"",$U35,IF($P35&lt;&gt;"",$P35,""))))),"")</f>
         <v/>
       </c>
       <c r="AP38" s="240" t="inlineStr">
         <is>
-          <t>Field/column completeness check — auto-derived (xem generate.md Step 3b)</t>
+          <t>Đối chứng phân biệt phạm vi OPR-05: cấm ở tầng NÚT HÀNH ĐỘNG, không phải ẩn tin khỏi danh sách (xem Analyst Note Block "Danh sách tin đăng", test_scenario_map.md)</t>
         </is>
       </c>
     </row>
@@ -5609,12 +5668,12 @@
       </c>
       <c r="B39" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-002</t>
+          <t>REQ-ASN-004</t>
         </is>
       </c>
       <c r="C39" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §A5 (BR-CON-01/02) + DOC-v1.0-02 §4.2</t>
+          <t>DOC-v1.0-01 §D3/§D4 (MTCH-01, BR-MTCH-01)</t>
         </is>
       </c>
       <c r="D39" s="239" t="inlineStr">
@@ -5629,24 +5688,24 @@
       </c>
       <c r="F39" s="239" t="inlineStr">
         <is>
-          <t>Check bấm "Huỷ" trong modal xác nhận → đóng modal, đơn KHÔNG đổi trạng thái</t>
+          <t>Check Carrier bấm "Nhận giao" từ thông báo khớp tuyến → đơn chuyển "Đã ghép"</t>
         </is>
       </c>
       <c r="G39" s="239" t="inlineStr">
         <is>
-          <t>Modal "Xác nhận mang giúp" đang mở trên 1 tin "Chờ ghép"</t>
+          <t>Carrier đã đăng tuyến OFFER và vừa nhận thông báo khớp tuyến về 1 tin NEED phù hợp</t>
         </is>
       </c>
       <c r="H39" s="239" t="inlineStr">
         <is>
-          <t>1. Mở app FoxEco
-2. Bấm tab "Bảng tin", mở Chi tiết tin của 1 tin "Chờ ghép", bấm "Tôi mang giúp được"
-3. Bấm nút "Huỷ" trong modal</t>
+          <t>1. Mở app FoxEco bằng tài khoản Carrier, mở màn Thông báo
+2. Bấm thông báo khớp tuyến để mở Chi tiết tin của tin NEED phù hợp
+3. Bấm "Nhận giao" và xác nhận</t>
         </is>
       </c>
       <c r="I39" s="239" t="inlineStr">
         <is>
-          <t>3. Modal đóng lại, quay về màn Chi tiết tin; đơn giữ nguyên trạng thái "Chờ ghép", SĐT hai bên KHÔNG bị lộ</t>
+          <t>3. Đơn chuyển sang trạng thái "Đã ghép", liên hệ 2 bên được lộ và Carrier vào được màn Theo dõi đơn</t>
         </is>
       </c>
       <c r="J39" s="239" t="inlineStr">
@@ -5691,128 +5750,70 @@
       <c r="AK39" s="240" t="n"/>
       <c r="AL39" s="240" t="n"/>
       <c r="AM39" s="241">
-        <f>IF($A39="","",IF(OR($N39="Yes",$S39="Yes",$X39="Yes",$AC39="Yes",$AH39="Yes"),"Yes","No"))</f>
+        <f>IF($A36="","",IF(OR($N36="Yes",$S36="Yes",$X36="Yes",$AC36="Yes",$AH36="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN39" s="241">
-        <f>IF($A39="","",IFERROR(IF($AI39&lt;&gt;"",$AI39,IF($AD39&lt;&gt;"",$AD39,IF($Y39&lt;&gt;"",$Y39,IF($T39&lt;&gt;"",$T39,IF($O39&lt;&gt;"",$O39,""))))),""))</f>
+        <f>IF($A36="","",IFERROR(IF($AI36&lt;&gt;"",$AI36,IF($AD36&lt;&gt;"",$AD36,IF($Y36&lt;&gt;"",$Y36,IF($T36&lt;&gt;"",$T36,IF($O36&lt;&gt;"",$O36,""))))),""))</f>
         <v/>
       </c>
       <c r="AO39" s="241">
-        <f>IFERROR(IF($AJ39&lt;&gt;"",$AJ39,IF($AE39&lt;&gt;"",$AE39,IF($Z39&lt;&gt;"",$Z39,IF($U39&lt;&gt;"",$U39,IF($P39&lt;&gt;"",$P39,""))))),"")</f>
+        <f>IFERROR(IF($AJ36&lt;&gt;"",$AJ36,IF($AE36&lt;&gt;"",$AE36,IF($Z36&lt;&gt;"",$Z36,IF($U36&lt;&gt;"",$U36,IF($P36&lt;&gt;"",$P36,""))))),"")</f>
         <v/>
       </c>
       <c r="AP39" s="240" t="inlineStr">
         <is>
-          <t>Technique: EP-cancel (partition không xác nhận)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="60" customHeight="1" s="206">
-      <c r="A40" s="239">
-        <f>IF(C40="","",$C$2&amp;"."&amp;COUNTA($C$8:C40)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="B40" s="239" t="inlineStr">
-        <is>
-          <t>REQ-ASN-002</t>
-        </is>
-      </c>
-      <c r="C40" s="239" t="inlineStr">
-        <is>
-          <t>DOC-v1.0-01 §A5 (BR-CON-01/02) + DOC-v1.0-02 §4.2</t>
-        </is>
-      </c>
-      <c r="D40" s="239" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="E40" s="239" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F40" s="239" t="inlineStr">
-        <is>
-          <t>Check bấm "Xác nhận" trong modal → đơn chuyển "Đã ghép" ngay, không cần chủ tin duyệt</t>
-        </is>
-      </c>
-      <c r="G40" s="239" t="inlineStr">
-        <is>
-          <t>Modal "Xác nhận mang giúp" đang mở trên 1 tin "Chờ ghép"</t>
-        </is>
-      </c>
-      <c r="H40" s="239" t="inlineStr">
-        <is>
-          <t>1. Mở app FoxEco bằng tài khoản Carrier
-2. Bấm tab "Bảng tin", mở Chi tiết tin của 1 tin "Chờ ghép", bấm "Tôi mang giúp được"
-3. Bấm nút "Xác nhận" trong modal</t>
-        </is>
-      </c>
-      <c r="I40" s="239" t="inlineStr">
-        <is>
-          <t>3. Đơn chuyển sang trạng thái "Đã ghép" NGAY lập tức, không phát sinh bước chờ chủ tin duyệt</t>
-        </is>
-      </c>
-      <c r="J40" s="239" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="K40" s="239" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L40" s="239" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M40" s="239" t="n"/>
-      <c r="N40" s="239" t="n"/>
-      <c r="O40" s="239" t="n"/>
-      <c r="P40" s="239" t="n"/>
-      <c r="Q40" s="239" t="n"/>
-      <c r="R40" s="239" t="n"/>
-      <c r="S40" s="239" t="n"/>
-      <c r="T40" s="239" t="n"/>
-      <c r="U40" s="239" t="n"/>
-      <c r="V40" s="239" t="n"/>
-      <c r="W40" s="239" t="n"/>
-      <c r="X40" s="239" t="n"/>
-      <c r="Y40" s="239" t="n"/>
-      <c r="Z40" s="239" t="n"/>
-      <c r="AA40" s="239" t="n"/>
-      <c r="AB40" s="240" t="n"/>
-      <c r="AC40" s="240" t="n"/>
-      <c r="AD40" s="240" t="n"/>
-      <c r="AE40" s="240" t="n"/>
-      <c r="AF40" s="240" t="n"/>
-      <c r="AG40" s="240" t="n"/>
-      <c r="AH40" s="240" t="n"/>
-      <c r="AI40" s="240" t="n"/>
-      <c r="AJ40" s="240" t="n"/>
-      <c r="AK40" s="240" t="n"/>
-      <c r="AL40" s="240" t="n"/>
-      <c r="AM40" s="241">
-        <f>IF($A40="","",IF(OR($N40="Yes",$S40="Yes",$X40="Yes",$AC40="Yes",$AH40="Yes"),"Yes","No"))</f>
-        <v/>
-      </c>
-      <c r="AN40" s="241">
-        <f>IF($A40="","",IFERROR(IF($AI40&lt;&gt;"",$AI40,IF($AD40&lt;&gt;"",$AD40,IF($Y40&lt;&gt;"",$Y40,IF($T40&lt;&gt;"",$T40,IF($O40&lt;&gt;"",$O40,""))))),""))</f>
-        <v/>
-      </c>
-      <c r="AO40" s="241">
-        <f>IFERROR(IF($AJ40&lt;&gt;"",$AJ40,IF($AE40&lt;&gt;"",$AE40,IF($Z40&lt;&gt;"",$Z40,IF($U40&lt;&gt;"",$U40,IF($P40&lt;&gt;"",$P40,""))))),"")</f>
-        <v/>
-      </c>
-      <c r="AP40" s="240" t="inlineStr">
-        <is>
-          <t>Technique: ST-posted-matched (transition tại modal xác nhận) | EP-confirm (partition xác nhận, cặp với EP-cancel)</t>
-        </is>
-      </c>
+          <t>⚠ Thuộc nhánh auto-match tuyến OFFER↔NEED — `Project_rule.md` Phase 1 Scope liệt kê nhánh này là NGOÀI phạm vi Phase 1 (PM chưa trả lời dứt điểm). Giữ TC để không mất coverage `SC-ASN-007`, đánh dấu chờ PM chốt scope trước khi đưa vào vòng chạy</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1" s="206">
+      <c r="A40" s="231" t="n"/>
+      <c r="B40" s="232" t="inlineStr">
+        <is>
+          <t>Block Modal xác nhận mang giúp</t>
+        </is>
+      </c>
+      <c r="C40" s="211" t="n"/>
+      <c r="D40" s="211" t="n"/>
+      <c r="E40" s="211" t="n"/>
+      <c r="F40" s="211" t="n"/>
+      <c r="G40" s="211" t="n"/>
+      <c r="H40" s="211" t="n"/>
+      <c r="I40" s="209" t="n"/>
+      <c r="J40" s="231" t="n"/>
+      <c r="K40" s="231" t="n"/>
+      <c r="L40" s="231" t="n"/>
+      <c r="M40" s="231" t="n"/>
+      <c r="N40" s="235" t="n"/>
+      <c r="O40" s="235" t="n"/>
+      <c r="P40" s="235" t="n"/>
+      <c r="Q40" s="235" t="n"/>
+      <c r="R40" s="235" t="n"/>
+      <c r="S40" s="235" t="n"/>
+      <c r="T40" s="235" t="n"/>
+      <c r="U40" s="235" t="n"/>
+      <c r="V40" s="235" t="n"/>
+      <c r="W40" s="235" t="n"/>
+      <c r="X40" s="235" t="n"/>
+      <c r="Y40" s="235" t="n"/>
+      <c r="Z40" s="235" t="n"/>
+      <c r="AA40" s="235" t="n"/>
+      <c r="AB40" s="236" t="n"/>
+      <c r="AC40" s="236" t="n"/>
+      <c r="AD40" s="236" t="n"/>
+      <c r="AE40" s="236" t="n"/>
+      <c r="AF40" s="236" t="n"/>
+      <c r="AG40" s="236" t="n"/>
+      <c r="AH40" s="236" t="n"/>
+      <c r="AI40" s="236" t="n"/>
+      <c r="AJ40" s="236" t="n"/>
+      <c r="AK40" s="236" t="n"/>
+      <c r="AL40" s="236" t="n"/>
+      <c r="AM40" s="237" t="n"/>
+      <c r="AN40" s="237" t="n"/>
+      <c r="AO40" s="237" t="n"/>
+      <c r="AP40" s="238" t="n"/>
     </row>
     <row r="41" ht="60" customHeight="1" s="206">
       <c r="A41" s="239">
@@ -5831,34 +5832,34 @@
       </c>
       <c r="D41" s="239" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E41" s="239" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F41" s="239" t="inlineStr">
         <is>
-          <t>Check SĐT hai bên được lộ và nút "Gọi" khả dụng ngay sau khi ghép</t>
+          <t>Check đầy đủ + đúng 3 thành phần hiển thị tại modal "Xác nhận mang giúp"</t>
         </is>
       </c>
       <c r="G41" s="239" t="inlineStr">
         <is>
-          <t>1 đơn vừa chuyển sang trạng thái "Đã ghép" (Carrier vừa bấm Xác nhận)</t>
+          <t>Đang ở Chi tiết tin của 1 tin "Chờ ghép", đã bấm nút "Tôi mang giúp được"</t>
         </is>
       </c>
       <c r="H41" s="239" t="inlineStr">
         <is>
-          <t>1. Trên thiết bị Carrier: sau khi ghép, mở lại màn chi tiết/theo dõi của đơn vừa ghép
-2. Quan sát phần liên hệ của Người gửi
-3. Đổi sang thiết bị Sender, mở đơn tương ứng và quan sát phần liên hệ của Carrier</t>
+          <t>1. Mở app FoxEco
+2. Bấm tab "Bảng tin", mở Chi tiết tin của 1 tin "Chờ ghép"
+3. Bấm "Tôi mang giúp được" và quan sát modal vừa hiện</t>
         </is>
       </c>
       <c r="I41" s="239" t="inlineStr">
         <is>
-          <t>3. Cả 2 phía đều thấy SĐT của đối phương và nút "Gọi" khả dụng — đúng rule BR-CON-02 (chỉ lộ SAU khi ghép, và chỉ cho đúng 2 người trong cặp ghép)</t>
+          <t>3. Modal hiển thị đủ 3 thành phần: (1) nội dung cảnh báo SĐT hai bên sẽ được lộ sau khi xác nhận, (2) nút "Huỷ", (3) nút "Xác nhận"</t>
         </is>
       </c>
       <c r="J41" s="239" t="inlineStr">
@@ -5903,18 +5904,22 @@
       <c r="AK41" s="240" t="n"/>
       <c r="AL41" s="240" t="n"/>
       <c r="AM41" s="241">
-        <f>IF($A41="","",IF(OR($N41="Yes",$S41="Yes",$X41="Yes",$AC41="Yes",$AH41="Yes"),"Yes","No"))</f>
+        <f>IF($A38="","",IF(OR($N38="Yes",$S38="Yes",$X38="Yes",$AC38="Yes",$AH38="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN41" s="241">
-        <f>IF($A41="","",IFERROR(IF($AI41&lt;&gt;"",$AI41,IF($AD41&lt;&gt;"",$AD41,IF($Y41&lt;&gt;"",$Y41,IF($T41&lt;&gt;"",$T41,IF($O41&lt;&gt;"",$O41,""))))),""))</f>
+        <f>IF($A38="","",IFERROR(IF($AI38&lt;&gt;"",$AI38,IF($AD38&lt;&gt;"",$AD38,IF($Y38&lt;&gt;"",$Y38,IF($T38&lt;&gt;"",$T38,IF($O38&lt;&gt;"",$O38,""))))),""))</f>
         <v/>
       </c>
       <c r="AO41" s="241">
-        <f>IFERROR(IF($AJ41&lt;&gt;"",$AJ41,IF($AE41&lt;&gt;"",$AE41,IF($Z41&lt;&gt;"",$Z41,IF($U41&lt;&gt;"",$U41,IF($P41&lt;&gt;"",$P41,""))))),"")</f>
+        <f>IFERROR(IF($AJ38&lt;&gt;"",$AJ38,IF($AE38&lt;&gt;"",$AE38,IF($Z38&lt;&gt;"",$Z38,IF($U38&lt;&gt;"",$U38,IF($P38&lt;&gt;"",$P38,""))))),"")</f>
         <v/>
       </c>
-      <c r="AP41" s="240" t="n"/>
+      <c r="AP41" s="240" t="inlineStr">
+        <is>
+          <t>Field/column completeness check — auto-derived (xem generate.md Step 3b)</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="60" customHeight="1" s="206">
       <c r="A42" s="239">
@@ -5938,29 +5943,29 @@
       </c>
       <c r="E42" s="239" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F42" s="239" t="inlineStr">
         <is>
-          <t>Check cả 3 khung Người gửi/Người vận chuyển/Người nhận đổi trạng thái tức thời sau khi ghép</t>
+          <t>Check bấm "Huỷ" trong modal xác nhận → đóng modal, đơn KHÔNG đổi trạng thái</t>
         </is>
       </c>
       <c r="G42" s="239" t="inlineStr">
         <is>
-          <t>3 tài khoản Sender / Carrier / Receiver của cùng 1 đơn đang mở app đồng thời; đơn đang ở "Chờ ghép"</t>
+          <t>Modal "Xác nhận mang giúp" đang mở trên 1 tin "Chờ ghép"</t>
         </is>
       </c>
       <c r="H42" s="239" t="inlineStr">
         <is>
-          <t>1. Trên thiết bị Carrier: mở Chi tiết tin, bấm "Tôi mang giúp được" rồi "Xác nhận"
-2. Ngay sau đó quan sát màn đơn trên thiết bị Sender
-3. Ngay sau đó quan sát màn đơn trên thiết bị Receiver</t>
+          <t>1. Mở app FoxEco
+2. Bấm tab "Bảng tin", mở Chi tiết tin của 1 tin "Chờ ghép", bấm "Tôi mang giúp được"
+3. Bấm nút "Huỷ" trong modal</t>
         </is>
       </c>
       <c r="I42" s="239" t="inlineStr">
         <is>
-          <t>3. Cả 3 khung (Người gửi / Người vận chuyển / Người nhận) đều hiển thị trạng thái "Đã ghép" tức thời, không cần thao tác tải lại thủ công</t>
+          <t>3. Modal đóng lại, quay về màn Chi tiết tin; đơn giữ nguyên trạng thái "Chờ ghép", SĐT hai bên KHÔNG bị lộ</t>
         </is>
       </c>
       <c r="J42" s="239" t="inlineStr">
@@ -6005,18 +6010,22 @@
       <c r="AK42" s="240" t="n"/>
       <c r="AL42" s="240" t="n"/>
       <c r="AM42" s="241">
-        <f>IF($A42="","",IF(OR($N42="Yes",$S42="Yes",$X42="Yes",$AC42="Yes",$AH42="Yes"),"Yes","No"))</f>
+        <f>IF($A39="","",IF(OR($N39="Yes",$S39="Yes",$X39="Yes",$AC39="Yes",$AH39="Yes"),"Yes","No"))</f>
         <v/>
       </c>
       <c r="AN42" s="241">
-        <f>IF($A42="","",IFERROR(IF($AI42&lt;&gt;"",$AI42,IF($AD42&lt;&gt;"",$AD42,IF($Y42&lt;&gt;"",$Y42,IF($T42&lt;&gt;"",$T42,IF($O42&lt;&gt;"",$O42,""))))),""))</f>
+        <f>IF($A39="","",IFERROR(IF($AI39&lt;&gt;"",$AI39,IF($AD39&lt;&gt;"",$AD39,IF($Y39&lt;&gt;"",$Y39,IF($T39&lt;&gt;"",$T39,IF($O39&lt;&gt;"",$O39,""))))),""))</f>
         <v/>
       </c>
       <c r="AO42" s="241">
-        <f>IFERROR(IF($AJ42&lt;&gt;"",$AJ42,IF($AE42&lt;&gt;"",$AE42,IF($Z42&lt;&gt;"",$Z42,IF($U42&lt;&gt;"",$U42,IF($P42&lt;&gt;"",$P42,""))))),"")</f>
+        <f>IFERROR(IF($AJ39&lt;&gt;"",$AJ39,IF($AE39&lt;&gt;"",$AE39,IF($Z39&lt;&gt;"",$Z39,IF($U39&lt;&gt;"",$U39,IF($P39&lt;&gt;"",$P39,""))))),"")</f>
         <v/>
       </c>
-      <c r="AP42" s="240" t="n"/>
+      <c r="AP42" s="240" t="inlineStr">
+        <is>
+          <t>Technique: EP-cancel (partition không xác nhận)</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="60" customHeight="1" s="206">
       <c r="A43" s="239">
@@ -6025,12 +6034,12 @@
       </c>
       <c r="B43" s="239" t="inlineStr">
         <is>
-          <t>REQ-ASN-003</t>
+          <t>REQ-ASN-002</t>
         </is>
       </c>
       <c r="C43" s="239" t="inlineStr">
         <is>
-          <t>DOC-v1.0-01 §D3/§D7 (ASN-03, OPR-03)</t>
+          <t>DOC-v1.0-01 §A5 (BR-CON-01/02) + DOC-v1.0-02 §4.2</t>
         </is>
       </c>
       <c r="D43" s="239" t="inlineStr">
@@ -6045,24 +6054,24 @@
       </c>
       <c r="F43" s="239" t="inlineStr">
         <is>
-          <t>Check 2 Carrier bấm "Tôi mang giúp được" gần đồng thời → chỉ 1 người ghép thành công</t>
+          <t>Check bấm "Xác nhận" trong modal → đơn chuyển "Đã ghép" ngay, không cần chủ tin duyệt</t>
         </is>
       </c>
       <c r="G43" s="239" t="inlineStr">
         <is>
-          <t>2 tài khoản Carrier khác nhau cùng mở sẵn màn Chi tiết tin của CÙNG 1 tin đang "Chờ ghép"</t>
+          <t>Modal "Xác nhận mang giúp" đang mở trên 1 tin "Chờ ghép"</t>
         </is>
       </c>
       <c r="H43" s="239" t="inlineStr">
         <is>
-          <t>1. Trên cả 2 thiết bị Carrier: bấm "Tôi mang giúp được" để mở modal xác nhận
-2. Bấm "Xác nhận" trên cả 2 thiết bị gần như đồng thời
-3. Quan sát kết quả trên từng thiết bị</t>
+          <t>1. Mở app FoxEco bằng tài khoản Carrier
+2. Bấm tab "Bảng tin", mở Chi tiết tin của 1 tin "Chờ ghép", bấm "Tôi mang giúp được"
+3. Bấm nút "Xác nhận" trong modal</t>
         </is>
       </c>
       <c r="I43" s="239" t="inlineStr">
         <is>
-          <t>3. Chỉ 1 Carrier ghép thành công (đơn chuyển "Đã ghép" đúng 1 lần, không tạo 2 bản ghi ghép); Carrier còn lại nhận thông báo tin đã có người nhận và KHÔNG được ghép</t>
+          <t>3. Đơn chuyển sang trạng thái "Đã ghép" NGAY lập tức, không phát sinh bước chờ chủ tin duyệt</t>
         </is>
       </c>
       <c r="J43" s="239" t="inlineStr">
@@ -6107,154 +6116,332 @@
       <c r="AK43" s="240" t="n"/>
       <c r="AL43" s="240" t="n"/>
       <c r="AM43" s="241">
+        <f>IF($A40="","",IF(OR($N40="Yes",$S40="Yes",$X40="Yes",$AC40="Yes",$AH40="Yes"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="AN43" s="241">
+        <f>IF($A40="","",IFERROR(IF($AI40&lt;&gt;"",$AI40,IF($AD40&lt;&gt;"",$AD40,IF($Y40&lt;&gt;"",$Y40,IF($T40&lt;&gt;"",$T40,IF($O40&lt;&gt;"",$O40,""))))),""))</f>
+        <v/>
+      </c>
+      <c r="AO43" s="241">
+        <f>IFERROR(IF($AJ40&lt;&gt;"",$AJ40,IF($AE40&lt;&gt;"",$AE40,IF($Z40&lt;&gt;"",$Z40,IF($U40&lt;&gt;"",$U40,IF($P40&lt;&gt;"",$P40,""))))),"")</f>
+        <v/>
+      </c>
+      <c r="AP43" s="240" t="inlineStr">
+        <is>
+          <t>Technique: ST-posted-matched (transition tại modal xác nhận) | EP-confirm (partition xác nhận, cặp với EP-cancel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1" s="206">
+      <c r="A44" s="239">
+        <f>IF(C44="","",$C$2&amp;"."&amp;COUNTA($C$8:C44)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="B44" s="239" t="inlineStr">
+        <is>
+          <t>REQ-ASN-002</t>
+        </is>
+      </c>
+      <c r="C44" s="239" t="inlineStr">
+        <is>
+          <t>DOC-v1.0-01 §A5 (BR-CON-01/02) + DOC-v1.0-02 §4.2</t>
+        </is>
+      </c>
+      <c r="D44" s="239" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E44" s="239" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F44" s="239" t="inlineStr">
+        <is>
+          <t>Check SĐT hai bên được lộ và nút "Gọi" khả dụng ngay sau khi ghép</t>
+        </is>
+      </c>
+      <c r="G44" s="239" t="inlineStr">
+        <is>
+          <t>1 đơn vừa chuyển sang trạng thái "Đã ghép" (Carrier vừa bấm Xác nhận)</t>
+        </is>
+      </c>
+      <c r="H44" s="239" t="inlineStr">
+        <is>
+          <t>1. Trên thiết bị Carrier: sau khi ghép, mở lại màn chi tiết/theo dõi của đơn vừa ghép
+2. Quan sát phần liên hệ của Người gửi
+3. Đổi sang thiết bị Sender, mở đơn tương ứng và quan sát phần liên hệ của Carrier</t>
+        </is>
+      </c>
+      <c r="I44" s="239" t="inlineStr">
+        <is>
+          <t>3. Cả 2 phía đều thấy SĐT của đối phương và nút "Gọi" khả dụng — đúng rule BR-CON-02 (chỉ lộ SAU khi ghép, và chỉ cho đúng 2 người trong cặp ghép)</t>
+        </is>
+      </c>
+      <c r="J44" s="239" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="K44" s="239" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L44" s="239" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M44" s="239" t="n"/>
+      <c r="N44" s="239" t="n"/>
+      <c r="O44" s="239" t="n"/>
+      <c r="P44" s="239" t="n"/>
+      <c r="Q44" s="239" t="n"/>
+      <c r="R44" s="239" t="n"/>
+      <c r="S44" s="239" t="n"/>
+      <c r="T44" s="239" t="n"/>
+      <c r="U44" s="239" t="n"/>
+      <c r="V44" s="239" t="n"/>
+      <c r="W44" s="239" t="n"/>
+      <c r="X44" s="239" t="n"/>
+      <c r="Y44" s="239" t="n"/>
+      <c r="Z44" s="239" t="n"/>
+      <c r="AA44" s="239" t="n"/>
+      <c r="AB44" s="240" t="n"/>
+      <c r="AC44" s="240" t="n"/>
+      <c r="AD44" s="240" t="n"/>
+      <c r="AE44" s="240" t="n"/>
+      <c r="AF44" s="240" t="n"/>
+      <c r="AG44" s="240" t="n"/>
+      <c r="AH44" s="240" t="n"/>
+      <c r="AI44" s="240" t="n"/>
+      <c r="AJ44" s="240" t="n"/>
+      <c r="AK44" s="240" t="n"/>
+      <c r="AL44" s="240" t="n"/>
+      <c r="AM44" s="241">
+        <f>IF($A41="","",IF(OR($N41="Yes",$S41="Yes",$X41="Yes",$AC41="Yes",$AH41="Yes"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="AN44" s="241">
+        <f>IF($A41="","",IFERROR(IF($AI41&lt;&gt;"",$AI41,IF($AD41&lt;&gt;"",$AD41,IF($Y41&lt;&gt;"",$Y41,IF($T41&lt;&gt;"",$T41,IF($O41&lt;&gt;"",$O41,""))))),""))</f>
+        <v/>
+      </c>
+      <c r="AO44" s="241">
+        <f>IFERROR(IF($AJ41&lt;&gt;"",$AJ41,IF($AE41&lt;&gt;"",$AE41,IF($Z41&lt;&gt;"",$Z41,IF($U41&lt;&gt;"",$U41,IF($P41&lt;&gt;"",$P41,""))))),"")</f>
+        <v/>
+      </c>
+      <c r="AP44" s="240" t="n"/>
+    </row>
+    <row r="45" ht="60" customHeight="1" s="206">
+      <c r="A45" s="239">
+        <f>IF(C45="","",$C$2&amp;"."&amp;COUNTA($C$8:C45)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="B45" s="239" t="inlineStr">
+        <is>
+          <t>REQ-ASN-002</t>
+        </is>
+      </c>
+      <c r="C45" s="239" t="inlineStr">
+        <is>
+          <t>DOC-v1.0-01 §A5 (BR-CON-01/02) + DOC-v1.0-02 §4.2</t>
+        </is>
+      </c>
+      <c r="D45" s="239" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E45" s="239" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F45" s="239" t="inlineStr">
+        <is>
+          <t>Check cả 3 khung Người gửi/Người vận chuyển/Người nhận đổi trạng thái tức thời sau khi ghép</t>
+        </is>
+      </c>
+      <c r="G45" s="239" t="inlineStr">
+        <is>
+          <t>3 tài khoản Sender / Carrier / Receiver của cùng 1 đơn đang mở app đồng thời; đơn đang ở "Chờ ghép"</t>
+        </is>
+      </c>
+      <c r="H45" s="239" t="inlineStr">
+        <is>
+          <t>1. Trên thiết bị Carrier: mở Chi tiết tin, bấm "Tôi mang giúp được" rồi "Xác nhận"
+2. Ngay sau đó quan sát màn đơn trên thiết bị Sender
+3. Ngay sau đó quan sát màn đơn trên thiết bị Receiver</t>
+        </is>
+      </c>
+      <c r="I45" s="239" t="inlineStr">
+        <is>
+          <t>3. Cả 3 khung (Người gửi / Người vận chuyển / Người nhận) đều hiển thị trạng thái "Đã ghép" tức thời, không cần thao tác tải lại thủ công</t>
+        </is>
+      </c>
+      <c r="J45" s="239" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="K45" s="239" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L45" s="239" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M45" s="239" t="n"/>
+      <c r="N45" s="239" t="n"/>
+      <c r="O45" s="239" t="n"/>
+      <c r="P45" s="239" t="n"/>
+      <c r="Q45" s="239" t="n"/>
+      <c r="R45" s="239" t="n"/>
+      <c r="S45" s="239" t="n"/>
+      <c r="T45" s="239" t="n"/>
+      <c r="U45" s="239" t="n"/>
+      <c r="V45" s="239" t="n"/>
+      <c r="W45" s="239" t="n"/>
+      <c r="X45" s="239" t="n"/>
+      <c r="Y45" s="239" t="n"/>
+      <c r="Z45" s="239" t="n"/>
+      <c r="AA45" s="239" t="n"/>
+      <c r="AB45" s="240" t="n"/>
+      <c r="AC45" s="240" t="n"/>
+      <c r="AD45" s="240" t="n"/>
+      <c r="AE45" s="240" t="n"/>
+      <c r="AF45" s="240" t="n"/>
+      <c r="AG45" s="240" t="n"/>
+      <c r="AH45" s="240" t="n"/>
+      <c r="AI45" s="240" t="n"/>
+      <c r="AJ45" s="240" t="n"/>
+      <c r="AK45" s="240" t="n"/>
+      <c r="AL45" s="240" t="n"/>
+      <c r="AM45" s="241">
+        <f>IF($A42="","",IF(OR($N42="Yes",$S42="Yes",$X42="Yes",$AC42="Yes",$AH42="Yes"),"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="AN45" s="241">
+        <f>IF($A42="","",IFERROR(IF($AI42&lt;&gt;"",$AI42,IF($AD42&lt;&gt;"",$AD42,IF($Y42&lt;&gt;"",$Y42,IF($T42&lt;&gt;"",$T42,IF($O42&lt;&gt;"",$O42,""))))),""))</f>
+        <v/>
+      </c>
+      <c r="AO45" s="241">
+        <f>IFERROR(IF($AJ42&lt;&gt;"",$AJ42,IF($AE42&lt;&gt;"",$AE42,IF($Z42&lt;&gt;"",$Z42,IF($U42&lt;&gt;"",$U42,IF($P42&lt;&gt;"",$P42,""))))),"")</f>
+        <v/>
+      </c>
+      <c r="AP45" s="240" t="n"/>
+    </row>
+    <row r="46" ht="60" customHeight="1" s="206">
+      <c r="A46" s="239">
+        <f>IF(C46="","",$C$2&amp;"."&amp;COUNTA($C$8:C46)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="B46" s="239" t="inlineStr">
+        <is>
+          <t>REQ-ASN-003</t>
+        </is>
+      </c>
+      <c r="C46" s="239" t="inlineStr">
+        <is>
+          <t>DOC-v1.0-01 §D3/§D7 (ASN-03, OPR-03)</t>
+        </is>
+      </c>
+      <c r="D46" s="239" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E46" s="239" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F46" s="239" t="inlineStr">
+        <is>
+          <t>Check 2 Carrier bấm "Tôi mang giúp được" gần đồng thời → chỉ 1 người ghép thành công</t>
+        </is>
+      </c>
+      <c r="G46" s="239" t="inlineStr">
+        <is>
+          <t>2 tài khoản Carrier khác nhau cùng mở sẵn màn Chi tiết tin của CÙNG 1 tin đang "Chờ ghép"</t>
+        </is>
+      </c>
+      <c r="H46" s="239" t="inlineStr">
+        <is>
+          <t>1. Trên cả 2 thiết bị Carrier: bấm "Tôi mang giúp được" để mở modal xác nhận
+2. Bấm "Xác nhận" trên cả 2 thiết bị gần như đồng thời
+3. Quan sát kết quả trên từng thiết bị</t>
+        </is>
+      </c>
+      <c r="I46" s="239" t="inlineStr">
+        <is>
+          <t>3. Chỉ 1 Carrier ghép thành công (đơn chuyển "Đã ghép" đúng 1 lần, không tạo 2 bản ghi ghép); Carrier còn lại nhận thông báo tin đã có người nhận và KHÔNG được ghép</t>
+        </is>
+      </c>
+      <c r="J46" s="239" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="K46" s="239" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L46" s="239" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M46" s="239" t="n"/>
+      <c r="N46" s="239" t="n"/>
+      <c r="O46" s="239" t="n"/>
+      <c r="P46" s="239" t="n"/>
+      <c r="Q46" s="239" t="n"/>
+      <c r="R46" s="239" t="n"/>
+      <c r="S46" s="239" t="n"/>
+      <c r="T46" s="239" t="n"/>
+      <c r="U46" s="239" t="n"/>
+      <c r="V46" s="239" t="n"/>
+      <c r="W46" s="239" t="n"/>
+      <c r="X46" s="239" t="n"/>
+      <c r="Y46" s="239" t="n"/>
+      <c r="Z46" s="239" t="n"/>
+      <c r="AA46" s="239" t="n"/>
+      <c r="AB46" s="240" t="n"/>
+      <c r="AC46" s="240" t="n"/>
+      <c r="AD46" s="240" t="n"/>
+      <c r="AE46" s="240" t="n"/>
+      <c r="AF46" s="240" t="n"/>
+      <c r="AG46" s="240" t="n"/>
+      <c r="AH46" s="240" t="n"/>
+      <c r="AI46" s="240" t="n"/>
+      <c r="AJ46" s="240" t="n"/>
+      <c r="AK46" s="240" t="n"/>
+      <c r="AL46" s="240" t="n"/>
+      <c r="AM46" s="241">
         <f>IF($A43="","",IF(OR($N43="Yes",$S43="Yes",$X43="Yes",$AC43="Yes",$AH43="Yes"),"Yes","No"))</f>
         <v/>
       </c>
-      <c r="AN43" s="241">
+      <c r="AN46" s="241">
         <f>IF($A43="","",IFERROR(IF($AI43&lt;&gt;"",$AI43,IF($AD43&lt;&gt;"",$AD43,IF($Y43&lt;&gt;"",$Y43,IF($T43&lt;&gt;"",$T43,IF($O43&lt;&gt;"",$O43,""))))),""))</f>
         <v/>
       </c>
-      <c r="AO43" s="241">
+      <c r="AO46" s="241">
         <f>IFERROR(IF($AJ43&lt;&gt;"",$AJ43,IF($AE43&lt;&gt;"",$AE43,IF($Z43&lt;&gt;"",$Z43,IF($U43&lt;&gt;"",$U43,IF($P43&lt;&gt;"",$P43,""))))),"")</f>
         <v/>
       </c>
-      <c r="AP43" s="240" t="inlineStr">
+      <c r="AP46" s="240" t="inlineStr">
         <is>
           <t>Test integrity quan trọng nhất module (race condition / transaction lock) — cần chạy thủ công đa thiết bị, tham khảo `/vibe-multi`</t>
         </is>
       </c>
-    </row>
-    <row r="44" s="206">
-      <c r="A44" s="231" t="n"/>
-      <c r="B44" s="231" t="n"/>
-      <c r="C44" s="231" t="n"/>
-      <c r="D44" s="231" t="n"/>
-      <c r="E44" s="231" t="n"/>
-      <c r="F44" s="249" t="n"/>
-      <c r="G44" s="249" t="n"/>
-      <c r="H44" s="249" t="n"/>
-      <c r="I44" s="249" t="n"/>
-      <c r="J44" s="231" t="n"/>
-      <c r="K44" s="231" t="n"/>
-      <c r="L44" s="231" t="n"/>
-      <c r="M44" s="231" t="n"/>
-      <c r="N44" s="235" t="n"/>
-      <c r="O44" s="235" t="n"/>
-      <c r="P44" s="235" t="n"/>
-      <c r="Q44" s="235" t="n"/>
-      <c r="R44" s="235" t="n"/>
-      <c r="S44" s="235" t="n"/>
-      <c r="T44" s="235" t="n"/>
-      <c r="U44" s="235" t="n"/>
-      <c r="V44" s="235" t="n"/>
-      <c r="W44" s="235" t="n"/>
-      <c r="X44" s="235" t="n"/>
-      <c r="Y44" s="235" t="n"/>
-      <c r="Z44" s="235" t="n"/>
-      <c r="AA44" s="235" t="n"/>
-      <c r="AB44" s="236" t="n"/>
-      <c r="AC44" s="236" t="n"/>
-      <c r="AD44" s="236" t="n"/>
-      <c r="AE44" s="236" t="n"/>
-      <c r="AF44" s="236" t="n"/>
-      <c r="AG44" s="236" t="n"/>
-      <c r="AH44" s="236" t="n"/>
-      <c r="AI44" s="236" t="n"/>
-      <c r="AJ44" s="236" t="n"/>
-      <c r="AK44" s="236" t="n"/>
-      <c r="AL44" s="236" t="n"/>
-      <c r="AM44" s="237" t="n"/>
-      <c r="AN44" s="237" t="n"/>
-      <c r="AO44" s="237" t="n"/>
-      <c r="AP44" s="238" t="n"/>
-    </row>
-    <row r="45" s="206">
-      <c r="A45" s="231" t="n"/>
-      <c r="B45" s="231" t="n"/>
-      <c r="C45" s="231" t="n"/>
-      <c r="D45" s="231" t="n"/>
-      <c r="E45" s="231" t="n"/>
-      <c r="F45" s="249" t="n"/>
-      <c r="G45" s="249" t="n"/>
-      <c r="H45" s="249" t="n"/>
-      <c r="I45" s="249" t="n"/>
-      <c r="J45" s="231" t="n"/>
-      <c r="K45" s="231" t="n"/>
-      <c r="L45" s="231" t="n"/>
-      <c r="M45" s="231" t="n"/>
-      <c r="N45" s="235" t="n"/>
-      <c r="O45" s="235" t="n"/>
-      <c r="P45" s="235" t="n"/>
-      <c r="Q45" s="235" t="n"/>
-      <c r="R45" s="235" t="n"/>
-      <c r="S45" s="235" t="n"/>
-      <c r="T45" s="235" t="n"/>
-      <c r="U45" s="235" t="n"/>
-      <c r="V45" s="235" t="n"/>
-      <c r="W45" s="235" t="n"/>
-      <c r="X45" s="235" t="n"/>
-      <c r="Y45" s="235" t="n"/>
-      <c r="Z45" s="235" t="n"/>
-      <c r="AA45" s="235" t="n"/>
-      <c r="AB45" s="236" t="n"/>
-      <c r="AC45" s="236" t="n"/>
-      <c r="AD45" s="236" t="n"/>
-      <c r="AE45" s="236" t="n"/>
-      <c r="AF45" s="236" t="n"/>
-      <c r="AG45" s="236" t="n"/>
-      <c r="AH45" s="236" t="n"/>
-      <c r="AI45" s="236" t="n"/>
-      <c r="AJ45" s="236" t="n"/>
-      <c r="AK45" s="236" t="n"/>
-      <c r="AL45" s="236" t="n"/>
-      <c r="AM45" s="237" t="n"/>
-      <c r="AN45" s="237" t="n"/>
-      <c r="AO45" s="237" t="n"/>
-      <c r="AP45" s="238" t="n"/>
-    </row>
-    <row r="46" s="206">
-      <c r="A46" s="231" t="n"/>
-      <c r="B46" s="231" t="n"/>
-      <c r="C46" s="231" t="n"/>
-      <c r="D46" s="231" t="n"/>
-      <c r="E46" s="231" t="n"/>
-      <c r="F46" s="249" t="n"/>
-      <c r="G46" s="249" t="n"/>
-      <c r="H46" s="249" t="n"/>
-      <c r="I46" s="249" t="n"/>
-      <c r="J46" s="231" t="n"/>
-      <c r="K46" s="231" t="n"/>
-      <c r="L46" s="231" t="n"/>
-      <c r="M46" s="231" t="n"/>
-      <c r="N46" s="235" t="n"/>
-      <c r="O46" s="235" t="n"/>
-      <c r="P46" s="235" t="n"/>
-      <c r="Q46" s="235" t="n"/>
-      <c r="R46" s="235" t="n"/>
-      <c r="S46" s="235" t="n"/>
-      <c r="T46" s="235" t="n"/>
-      <c r="U46" s="235" t="n"/>
-      <c r="V46" s="235" t="n"/>
-      <c r="W46" s="235" t="n"/>
-      <c r="X46" s="235" t="n"/>
-      <c r="Y46" s="235" t="n"/>
-      <c r="Z46" s="235" t="n"/>
-      <c r="AA46" s="235" t="n"/>
-      <c r="AB46" s="236" t="n"/>
-      <c r="AC46" s="236" t="n"/>
-      <c r="AD46" s="236" t="n"/>
-      <c r="AE46" s="236" t="n"/>
-      <c r="AF46" s="236" t="n"/>
-      <c r="AG46" s="236" t="n"/>
-      <c r="AH46" s="236" t="n"/>
-      <c r="AI46" s="236" t="n"/>
-      <c r="AJ46" s="236" t="n"/>
-      <c r="AK46" s="236" t="n"/>
-      <c r="AL46" s="236" t="n"/>
-      <c r="AM46" s="237" t="n"/>
-      <c r="AN46" s="237" t="n"/>
-      <c r="AO46" s="237" t="n"/>
-      <c r="AP46" s="238" t="n"/>
     </row>
     <row r="47" s="206">
       <c r="A47" s="231" t="n"/>
@@ -20827,7 +21014,7 @@
   <autoFilter ref="A6:U6"/>
   <mergeCells count="25">
     <mergeCell ref="A7:I7"/>
-    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B22:I22"/>
     <mergeCell ref="AH5:AL5"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="A5:C5"/>
@@ -20839,18 +21026,18 @@
     <mergeCell ref="N5:R5"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B29:I29"/>
     <mergeCell ref="D5:I5"/>
+    <mergeCell ref="B28:I28"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="X5:AB5"/>
-    <mergeCell ref="B37:I37"/>
+    <mergeCell ref="B40:I40"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="AM5:AP5"/>
-    <mergeCell ref="B20:I20"/>
     <mergeCell ref="S5:W5"/>
     <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B32:I32"/>
   </mergeCells>
   <dataValidations count="8">
     <dataValidation sqref="J8:J17 J19:J502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
@@ -21105,7 +21292,7 @@
         </is>
       </c>
       <c r="L3" s="253" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M3" s="254" t="inlineStr">
         <is>
@@ -21698,6 +21885,71 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="253" t="inlineStr">
+        <is>
+          <t>SC-ORD-034</t>
+        </is>
+      </c>
+      <c r="B13" s="253" t="inlineStr">
+        <is>
+          <t>Icon quay lại tại màn Chi tiết tin</t>
+        </is>
+      </c>
+      <c r="C13" s="253" t="inlineStr">
+        <is>
+          <t>Quan sát thực tế app STG (QA GiangDC2, chat 2026-07-30)</t>
+        </is>
+      </c>
+      <c r="D13" s="255" t="inlineStr">
+        <is>
+          <t>N/A: display/navigation-only, không có input/condition để áp dụng technique</t>
+        </is>
+      </c>
+      <c r="E13" s="255" t="inlineStr">
+        <is>
+          <t>N/A: display/navigation-only, không có input/condition để áp dụng technique</t>
+        </is>
+      </c>
+      <c r="F13" s="255" t="inlineStr">
+        <is>
+          <t>N/A: display/navigation-only, không có input/condition để áp dụng technique</t>
+        </is>
+      </c>
+      <c r="G13" s="255" t="inlineStr">
+        <is>
+          <t>N/A: display/navigation-only, không có input/condition để áp dụng technique</t>
+        </is>
+      </c>
+      <c r="H13" s="255" t="inlineStr">
+        <is>
+          <t>N/A: display/navigation-only, không có input/condition để áp dụng technique</t>
+        </is>
+      </c>
+      <c r="I13" s="255" t="inlineStr">
+        <is>
+          <t>N/A: display/navigation-only, không có input/condition để áp dụng technique</t>
+        </is>
+      </c>
+      <c r="J13" s="255" t="inlineStr">
+        <is>
+          <t>N/A: display/navigation-only, không có input/condition để áp dụng technique</t>
+        </is>
+      </c>
+      <c r="K13" s="255" t="inlineStr">
+        <is>
+          <t>N/A: display/navigation-only, không có input/condition để áp dụng technique</t>
+        </is>
+      </c>
+      <c r="L13" s="253" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="257" t="inlineStr">
+        <is>
+          <t>N/A (0 applicable)</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
       <c r="A14" s="205" t="inlineStr">
         <is>
@@ -21708,7 +21960,7 @@
     <row r="15">
       <c r="A15" s="205" t="inlineStr">
         <is>
-          <t>Total TCs derived: 31</t>
+          <t>Total TCs derived: 34</t>
         </is>
       </c>
     </row>

</xml_diff>